<commit_message>
AWRI-127-60 list price 15,500 (confirmed)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDkGV31XDfJfqmsPKVkBWY
</commit_message>
<xml_diff>
--- a/pricing/ImpactCal_Pricelist_2026-09.xlsx
+++ b/pricing/ImpactCal_Pricelist_2026-09.xlsx
@@ -20693,7 +20693,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>product list / AWRI selector</t>
+          <t>confirmed by Paresh 24-09-2026</t>
         </is>
       </c>
       <c r="G62" t="n">
@@ -20703,7 +20703,7 @@
         <v>0</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>25000</v>
+        <v>15500</v>
       </c>
       <c r="J62">
         <f>IF(I62&gt;0,CEILING(I62*(1-Policy!$B$13/100),IF(I62&lt;10000,50,100)),"")</f>

</xml_diff>

<commit_message>
Prices: AWRI-127-60 Rs 15,500 confirmed; apply 2019/2018 price list (AD, AC-64, YSR)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDkGV31XDfJfqmsPKVkBWY
</commit_message>
<xml_diff>
--- a/pricing/ImpactCal_Pricelist_2026-09.xlsx
+++ b/pricing/ImpactCal_Pricelist_2026-09.xlsx
@@ -475,8 +475,6 @@
           <t>ADONI TECH — ImpactCal global price list &amp; costing</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -489,20 +487,14 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>PRICING POLICY (agreed 23-24 Sep 2026)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -515,7 +507,6 @@
           <t>Highest price found in any of the 8 uploaded price lists is taken as-is (list price).</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -528,7 +519,6 @@
           <t>Cost model per series (price ~ k · Fs^a · stroke^b fitted on your own prices; median error 6 % crane, 9 % industrial) + negotiation margin below</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -541,7 +531,6 @@
           <t>Moulding cost + hardware + mould cost amortised, + margin over cost (parameters below; Rubber mounts sheet recalculates live)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -554,7 +543,6 @@
           <t>nearest ₹50 below ₹10,000, nearest ₹100 above (always up)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -567,12 +555,8 @@
           <t>list ÷ live INR/USD rate × (1 + export uplift); recomputed at quotation time; column here is indicative</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -811,7 +795,6 @@
           <t>8 / 4 / 1</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1044,8 +1027,6 @@
           <t>blue = estimated value</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1385,11 +1366,11 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>980</v>
+        <v>1100</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>product_list:market</t>
+          <t>price list 2019 (Price List India 2022-23.pdf)</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -1399,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="J6">
         <f>IF(I6&gt;0,CEILING(I6*(1-Policy!$B$13/100),IF(I6&lt;10000,50,100)),"")</f>
@@ -1659,8 +1640,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" s="6" t="n">
         <v>3669</v>
       </c>
@@ -2530,19 +2509,25 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>11000</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G27" s="6" t="n">
         <v>13156</v>
       </c>
       <c r="H27" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>16500</v>
+        <v>11000</v>
       </c>
       <c r="J27">
         <f>IF(I27&gt;0,CEILING(I27*(1-Policy!$B$13/100),IF(I27&lt;10000,50,100)),"")</f>
@@ -2579,19 +2564,25 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>12500</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G28" s="6" t="n">
         <v>15556</v>
       </c>
       <c r="H28" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>19500</v>
+        <v>12500</v>
       </c>
       <c r="J28">
         <f>IF(I28&gt;0,CEILING(I28*(1-Policy!$B$13/100),IF(I28&lt;10000,50,100)),"")</f>
@@ -2631,8 +2622,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" s="6" t="n">
         <v>22637</v>
       </c>
@@ -2680,8 +2669,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" s="6" t="n">
         <v>22711</v>
       </c>
@@ -2729,8 +2716,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" s="6" t="n">
         <v>30472</v>
       </c>
@@ -2778,8 +2763,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" s="6" t="n">
         <v>32765</v>
       </c>
@@ -2827,8 +2810,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" s="6" t="n">
         <v>35158</v>
       </c>
@@ -2876,8 +2857,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" s="6" t="n">
         <v>4638</v>
       </c>
@@ -2925,8 +2904,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
       <c r="G35" s="6" t="n">
         <v>4638</v>
       </c>
@@ -2974,8 +2951,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" s="6" t="n">
         <v>6578</v>
       </c>
@@ -3078,8 +3053,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" s="6" t="n">
         <v>8783</v>
       </c>
@@ -3127,8 +3100,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
       <c r="G39" s="6" t="n">
         <v>12227</v>
       </c>
@@ -3176,8 +3147,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
       <c r="G40" s="6" t="n">
         <v>14740</v>
       </c>
@@ -3225,8 +3194,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
       <c r="G41" s="6" t="n">
         <v>16533</v>
       </c>
@@ -3275,11 +3242,11 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1300</v>
+        <v>1400</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>product_list:b2b</t>
+          <t>price list 2019 (Price List India 2022-23.pdf)</t>
         </is>
       </c>
       <c r="G42" t="n">
@@ -3289,7 +3256,7 @@
         <v>0</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>1300</v>
+        <v>1400</v>
       </c>
       <c r="J42">
         <f>IF(I42&gt;0,CEILING(I42*(1-Policy!$B$13/100),IF(I42&lt;10000,50,100)),"")</f>
@@ -3330,11 +3297,11 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>2200</v>
+        <v>2400</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>product_list:market</t>
+          <t>price list 2019 (Price List India 2022-23.pdf)</t>
         </is>
       </c>
       <c r="G43" t="n">
@@ -3344,7 +3311,7 @@
         <v>0</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>2200</v>
+        <v>2400</v>
       </c>
       <c r="J43">
         <f>IF(I43&gt;0,CEILING(I43*(1-Policy!$B$13/100),IF(I43&lt;10000,50,100)),"")</f>
@@ -3494,8 +3461,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" s="6" t="n">
         <v>4235</v>
       </c>
@@ -4145,19 +4110,25 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G58" s="6" t="n">
         <v>7701</v>
       </c>
       <c r="H58" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>9650</v>
+        <v>8500</v>
       </c>
       <c r="J58">
         <f>IF(I58&gt;0,CEILING(I58*(1-Policy!$B$13/100),IF(I58&lt;10000,50,100)),"")</f>
@@ -4249,19 +4220,25 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>11800</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G60" s="6" t="n">
         <v>9296</v>
       </c>
       <c r="H60" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>11700</v>
+        <v>11800</v>
       </c>
       <c r="J60">
         <f>IF(I60&gt;0,CEILING(I60*(1-Policy!$B$13/100),IF(I60&lt;10000,50,100)),"")</f>
@@ -4298,19 +4275,25 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G61" s="6" t="n">
         <v>10378</v>
       </c>
       <c r="H61" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I61" s="3" t="n">
-        <v>13000</v>
+        <v>12000</v>
       </c>
       <c r="J61">
         <f>IF(I61&gt;0,CEILING(I61*(1-Policy!$B$13/100),IF(I61&lt;10000,50,100)),"")</f>
@@ -4347,19 +4330,25 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G62" s="6" t="n">
         <v>14212</v>
       </c>
       <c r="H62" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>17800</v>
+        <v>15000</v>
       </c>
       <c r="J62">
         <f>IF(I62&gt;0,CEILING(I62*(1-Policy!$B$13/100),IF(I62&lt;10000,50,100)),"")</f>
@@ -4396,19 +4385,25 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>17500</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G63" s="6" t="n">
         <v>16805</v>
       </c>
       <c r="H63" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>21100</v>
+        <v>17500</v>
       </c>
       <c r="J63">
         <f>IF(I63&gt;0,CEILING(I63*(1-Policy!$B$13/100),IF(I63&lt;10000,50,100)),"")</f>
@@ -4503,8 +4498,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
       <c r="G65" s="6" t="n">
         <v>40131</v>
       </c>
@@ -4549,19 +4542,25 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>44000</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G66" s="6" t="n">
         <v>32918</v>
       </c>
       <c r="H66" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>41200</v>
+        <v>44000</v>
       </c>
       <c r="J66">
         <f>IF(I66&gt;0,CEILING(I66*(1-Policy!$B$13/100),IF(I66&lt;10000,50,100)),"")</f>
@@ -4598,19 +4597,25 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>50000</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G67" s="6" t="n">
         <v>35395</v>
       </c>
       <c r="H67" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I67" s="3" t="n">
-        <v>44300</v>
+        <v>50000</v>
       </c>
       <c r="J67">
         <f>IF(I67&gt;0,CEILING(I67*(1-Policy!$B$13/100),IF(I67&lt;10000,50,100)),"")</f>
@@ -4647,19 +4652,25 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>55000</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G68" s="6" t="n">
         <v>37981</v>
       </c>
       <c r="H68" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>47500</v>
+        <v>55000</v>
       </c>
       <c r="J68">
         <f>IF(I68&gt;0,CEILING(I68*(1-Policy!$B$13/100),IF(I68&lt;10000,50,100)),"")</f>
@@ -4919,8 +4930,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" s="6" t="n">
         <v>20689</v>
       </c>
@@ -5353,8 +5362,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
       <c r="G81" s="6" t="n">
         <v>26890</v>
       </c>
@@ -5897,8 +5904,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
-      <c r="F91" t="inlineStr"/>
       <c r="G91" s="6" t="n">
         <v>52785</v>
       </c>
@@ -5946,8 +5951,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="inlineStr"/>
       <c r="G92" s="6" t="n">
         <v>60795</v>
       </c>
@@ -5995,8 +5998,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
-      <c r="F93" t="inlineStr"/>
       <c r="G93" s="6" t="n">
         <v>68832</v>
       </c>
@@ -6264,8 +6265,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr"/>
       <c r="G98" s="6" t="n">
         <v>58913</v>
       </c>
@@ -6313,8 +6312,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr"/>
       <c r="G99" s="6" t="n">
         <v>69090</v>
       </c>
@@ -6527,8 +6524,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr"/>
       <c r="G103" s="6" t="n">
         <v>70653</v>
       </c>
@@ -6741,8 +6736,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr"/>
       <c r="G107" s="6" t="n">
         <v>81211</v>
       </c>
@@ -6955,8 +6948,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
       <c r="G111" s="6" t="n">
         <v>73543</v>
       </c>
@@ -7059,8 +7050,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
       <c r="G113" s="6" t="n">
         <v>85653</v>
       </c>
@@ -7493,8 +7482,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr"/>
       <c r="G121" s="6" t="n">
         <v>89371</v>
       </c>
@@ -7542,8 +7529,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" s="6" t="n">
         <v>80189</v>
       </c>
@@ -7701,8 +7686,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr"/>
       <c r="G125" s="6" t="n">
         <v>81294</v>
       </c>
@@ -7805,8 +7788,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr"/>
       <c r="G127" s="6" t="n">
         <v>94259</v>
       </c>
@@ -7909,8 +7890,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
-      <c r="F129" t="inlineStr"/>
       <c r="G129" s="6" t="n">
         <v>80100</v>
       </c>
@@ -7958,8 +7937,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
-      <c r="F130" t="inlineStr"/>
       <c r="G130" s="6" t="n">
         <v>79673</v>
       </c>
@@ -8007,8 +7984,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
-      <c r="F131" t="inlineStr"/>
       <c r="G131" s="6" t="n">
         <v>99666</v>
       </c>
@@ -8056,8 +8031,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
-      <c r="F132" t="inlineStr"/>
       <c r="G132" s="6" t="n">
         <v>106423</v>
       </c>
@@ -8105,8 +8078,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
-      <c r="F133" t="inlineStr"/>
       <c r="G133" s="6" t="n">
         <v>112858</v>
       </c>
@@ -8209,8 +8180,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
-      <c r="F135" t="inlineStr"/>
       <c r="G135" s="6" t="n">
         <v>29935</v>
       </c>
@@ -8258,8 +8227,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
-      <c r="F136" t="inlineStr"/>
       <c r="G136" s="6" t="n">
         <v>31513</v>
       </c>
@@ -8307,8 +8274,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
-      <c r="F137" t="inlineStr"/>
       <c r="G137" s="6" t="n">
         <v>42694</v>
       </c>
@@ -8356,8 +8321,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
-      <c r="F138" t="inlineStr"/>
       <c r="G138" s="6" t="n">
         <v>49521</v>
       </c>
@@ -8405,8 +8368,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
-      <c r="F139" t="inlineStr"/>
       <c r="G139" s="6" t="n">
         <v>45237</v>
       </c>
@@ -8454,8 +8415,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
-      <c r="F140" t="inlineStr"/>
       <c r="G140" s="6" t="n">
         <v>55448</v>
       </c>
@@ -8503,8 +8462,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
-      <c r="F141" t="inlineStr"/>
       <c r="G141" s="6" t="n">
         <v>15625</v>
       </c>
@@ -8552,8 +8509,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
-      <c r="F142" t="inlineStr"/>
       <c r="G142" s="6" t="n">
         <v>17980</v>
       </c>
@@ -8601,8 +8556,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
-      <c r="F143" t="inlineStr"/>
       <c r="G143" s="6" t="n">
         <v>19750</v>
       </c>
@@ -8650,8 +8603,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr"/>
-      <c r="F144" t="inlineStr"/>
       <c r="G144" s="6" t="n">
         <v>27713</v>
       </c>
@@ -8699,8 +8650,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr"/>
       <c r="G145" s="6" t="n">
         <v>21214</v>
       </c>
@@ -8748,8 +8697,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr"/>
-      <c r="F146" t="inlineStr"/>
       <c r="G146" s="6" t="n">
         <v>32461</v>
       </c>
@@ -8797,8 +8744,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr"/>
-      <c r="F147" t="inlineStr"/>
       <c r="G147" s="6" t="n">
         <v>30749</v>
       </c>
@@ -8846,8 +8791,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
-      <c r="F148" t="inlineStr"/>
       <c r="G148" s="6" t="n">
         <v>22335</v>
       </c>
@@ -8895,8 +8838,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr"/>
-      <c r="F149" t="inlineStr"/>
       <c r="G149" s="6" t="n">
         <v>35819</v>
       </c>
@@ -8944,8 +8885,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
-      <c r="F150" t="inlineStr"/>
       <c r="G150" s="6" t="n">
         <v>27425</v>
       </c>
@@ -8993,8 +8932,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr"/>
-      <c r="F151" t="inlineStr"/>
       <c r="G151" s="6" t="n">
         <v>23369</v>
       </c>
@@ -9042,8 +8979,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr"/>
-      <c r="F152" t="inlineStr"/>
       <c r="G152" s="6" t="n">
         <v>23976</v>
       </c>
@@ -9091,8 +9026,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr"/>
-      <c r="F153" t="inlineStr"/>
       <c r="G153" s="6" t="n">
         <v>29404</v>
       </c>
@@ -9140,8 +9073,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr"/>
-      <c r="F154" t="inlineStr"/>
       <c r="G154" s="6" t="n">
         <v>24434</v>
       </c>
@@ -9189,8 +9120,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
-      <c r="F155" t="inlineStr"/>
       <c r="G155" s="6" t="n">
         <v>34635</v>
       </c>
@@ -9238,8 +9167,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr"/>
-      <c r="F156" t="inlineStr"/>
       <c r="G156" s="6" t="n">
         <v>24670</v>
       </c>
@@ -9287,8 +9214,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr"/>
-      <c r="F157" t="inlineStr"/>
       <c r="G157" s="6" t="n">
         <v>38300</v>
       </c>
@@ -9336,8 +9261,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr"/>
-      <c r="F158" t="inlineStr"/>
       <c r="G158" s="6" t="n">
         <v>24867</v>
       </c>
@@ -9385,8 +9308,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr"/>
-      <c r="F159" t="inlineStr"/>
       <c r="G159" s="6" t="n">
         <v>31172</v>
       </c>
@@ -9434,8 +9355,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr"/>
-      <c r="F160" t="inlineStr"/>
       <c r="G160" s="6" t="n">
         <v>25070</v>
       </c>
@@ -9483,8 +9402,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E161" t="inlineStr"/>
-      <c r="F161" t="inlineStr"/>
       <c r="G161" s="6" t="n">
         <v>42121</v>
       </c>
@@ -9532,8 +9449,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr"/>
-      <c r="F162" t="inlineStr"/>
       <c r="G162" s="6" t="n">
         <v>25112</v>
       </c>
@@ -9581,8 +9496,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr"/>
-      <c r="F163" t="inlineStr"/>
       <c r="G163" s="6" t="n">
         <v>32430</v>
       </c>
@@ -9630,8 +9543,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr"/>
-      <c r="F164" t="inlineStr"/>
       <c r="G164" s="6" t="n">
         <v>37139</v>
       </c>
@@ -9679,8 +9590,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr"/>
-      <c r="F165" t="inlineStr"/>
       <c r="G165" s="6" t="n">
         <v>25264</v>
       </c>
@@ -9728,8 +9637,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr"/>
-      <c r="F166" t="inlineStr"/>
       <c r="G166" s="6" t="n">
         <v>33063</v>
       </c>
@@ -9777,8 +9684,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr"/>
-      <c r="F167" t="inlineStr"/>
       <c r="G167" s="6" t="n">
         <v>42077</v>
       </c>
@@ -9826,8 +9731,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E168" t="inlineStr"/>
-      <c r="F168" t="inlineStr"/>
       <c r="G168" s="6" t="n">
         <v>33717</v>
       </c>
@@ -9875,8 +9778,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E169" t="inlineStr"/>
-      <c r="F169" t="inlineStr"/>
       <c r="G169" s="6" t="n">
         <v>38513</v>
       </c>
@@ -9924,8 +9825,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E170" t="inlineStr"/>
-      <c r="F170" t="inlineStr"/>
       <c r="G170" s="6" t="n">
         <v>46129</v>
       </c>
@@ -9973,8 +9872,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E171" t="inlineStr"/>
-      <c r="F171" t="inlineStr"/>
       <c r="G171" s="6" t="n">
         <v>34304</v>
       </c>
@@ -10022,8 +9919,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E172" t="inlineStr"/>
-      <c r="F172" t="inlineStr"/>
       <c r="G172" s="6" t="n">
         <v>39761</v>
       </c>
@@ -10071,8 +9966,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E173" t="inlineStr"/>
-      <c r="F173" t="inlineStr"/>
       <c r="G173" s="6" t="n">
         <v>44687</v>
       </c>
@@ -10120,8 +10013,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr"/>
-      <c r="F174" t="inlineStr"/>
       <c r="G174" s="6" t="n">
         <v>34832</v>
       </c>
@@ -10169,8 +10060,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr"/>
-      <c r="F175" t="inlineStr"/>
       <c r="G175" s="6" t="n">
         <v>35928</v>
       </c>
@@ -10218,8 +10107,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E176" t="inlineStr"/>
-      <c r="F176" t="inlineStr"/>
       <c r="G176" s="6" t="n">
         <v>46027</v>
       </c>
@@ -10267,8 +10154,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E177" t="inlineStr"/>
-      <c r="F177" t="inlineStr"/>
       <c r="G177" s="6" t="n">
         <v>49530</v>
       </c>
@@ -10316,8 +10201,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr"/>
-      <c r="F178" t="inlineStr"/>
       <c r="G178" s="6" t="n">
         <v>42595</v>
       </c>
@@ -10365,8 +10248,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr"/>
-      <c r="F179" t="inlineStr"/>
       <c r="G179" s="6" t="n">
         <v>36962</v>
       </c>
@@ -10414,8 +10295,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr"/>
-      <c r="F180" t="inlineStr"/>
       <c r="G180" s="6" t="n">
         <v>43498</v>
       </c>
@@ -10463,8 +10342,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr"/>
-      <c r="F181" t="inlineStr"/>
       <c r="G181" s="6" t="n">
         <v>35830</v>
       </c>
@@ -10512,8 +10389,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr"/>
-      <c r="F182" t="inlineStr"/>
       <c r="G182" s="6" t="n">
         <v>47326</v>
       </c>
@@ -10561,8 +10436,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr"/>
-      <c r="F183" t="inlineStr"/>
       <c r="G183" s="6" t="n">
         <v>52098</v>
       </c>
@@ -10610,8 +10483,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr"/>
-      <c r="F184" t="inlineStr"/>
       <c r="G184" s="6" t="n">
         <v>44353</v>
       </c>
@@ -10659,8 +10530,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E185" t="inlineStr"/>
-      <c r="F185" t="inlineStr"/>
       <c r="G185" s="6" t="n">
         <v>45164</v>
       </c>
@@ -10708,8 +10577,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E186" t="inlineStr"/>
-      <c r="F186" t="inlineStr"/>
       <c r="G186" s="6" t="n">
         <v>49586</v>
       </c>
@@ -10757,8 +10624,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E187" t="inlineStr"/>
-      <c r="F187" t="inlineStr"/>
       <c r="G187" s="6" t="n">
         <v>54439</v>
       </c>
@@ -10806,8 +10671,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E188" t="inlineStr"/>
-      <c r="F188" t="inlineStr"/>
       <c r="G188" s="6" t="n">
         <v>46646</v>
       </c>
@@ -10855,8 +10718,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E189" t="inlineStr"/>
-      <c r="F189" t="inlineStr"/>
       <c r="G189" s="6" t="n">
         <v>41784</v>
       </c>
@@ -10904,8 +10765,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E190" t="inlineStr"/>
-      <c r="F190" t="inlineStr"/>
       <c r="G190" s="6" t="n">
         <v>40599</v>
       </c>
@@ -10953,8 +10812,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr"/>
-      <c r="F191" t="inlineStr"/>
       <c r="G191" s="6" t="n">
         <v>41080</v>
       </c>
@@ -11002,8 +10859,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E192" t="inlineStr"/>
-      <c r="F192" t="inlineStr"/>
       <c r="G192" s="6" t="n">
         <v>48023</v>
       </c>
@@ -11051,8 +10906,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E193" t="inlineStr"/>
-      <c r="F193" t="inlineStr"/>
       <c r="G193" s="6" t="n">
         <v>53650</v>
       </c>
@@ -11100,8 +10953,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E194" t="inlineStr"/>
-      <c r="F194" t="inlineStr"/>
       <c r="G194" s="6" t="n">
         <v>58216</v>
       </c>
@@ -11149,8 +11000,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E195" t="inlineStr"/>
-      <c r="F195" t="inlineStr"/>
       <c r="G195" s="6" t="n">
         <v>41168</v>
       </c>
@@ -11198,8 +11047,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E196" t="inlineStr"/>
-      <c r="F196" t="inlineStr"/>
       <c r="G196" s="6" t="n">
         <v>49268</v>
       </c>
@@ -11247,8 +11094,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E197" t="inlineStr"/>
-      <c r="F197" t="inlineStr"/>
       <c r="G197" s="6" t="n">
         <v>55239</v>
       </c>
@@ -11296,8 +11141,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E198" t="inlineStr"/>
-      <c r="F198" t="inlineStr"/>
       <c r="G198" s="6" t="n">
         <v>50893</v>
       </c>
@@ -11345,8 +11188,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E199" t="inlineStr"/>
-      <c r="F199" t="inlineStr"/>
       <c r="G199" s="6" t="n">
         <v>61426</v>
       </c>
@@ -11394,8 +11235,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E200" t="inlineStr"/>
-      <c r="F200" t="inlineStr"/>
       <c r="G200" s="6" t="n">
         <v>56693</v>
       </c>
@@ -11443,8 +11282,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr"/>
-      <c r="F201" t="inlineStr"/>
       <c r="G201" s="6" t="n">
         <v>51435</v>
       </c>
@@ -11492,8 +11329,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr"/>
-      <c r="F202" t="inlineStr"/>
       <c r="G202" s="6" t="n">
         <v>58064</v>
       </c>
@@ -11541,8 +11376,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E203" t="inlineStr"/>
-      <c r="F203" t="inlineStr"/>
       <c r="G203" s="6" t="n">
         <v>51967</v>
       </c>
@@ -11590,8 +11423,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E204" t="inlineStr"/>
-      <c r="F204" t="inlineStr"/>
       <c r="G204" s="6" t="n">
         <v>64157</v>
       </c>
@@ -11639,8 +11470,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E205" t="inlineStr"/>
-      <c r="F205" t="inlineStr"/>
       <c r="G205" s="6" t="n">
         <v>52150</v>
       </c>
@@ -11688,8 +11517,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E206" t="inlineStr"/>
-      <c r="F206" t="inlineStr"/>
       <c r="G206" s="6" t="n">
         <v>59346</v>
       </c>
@@ -11737,8 +11564,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E207" t="inlineStr"/>
-      <c r="F207" t="inlineStr"/>
       <c r="G207" s="6" t="n">
         <v>52495</v>
       </c>
@@ -11786,8 +11611,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr"/>
-      <c r="F208" t="inlineStr"/>
       <c r="G208" s="6" t="n">
         <v>66481</v>
       </c>
@@ -11835,8 +11658,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr"/>
-      <c r="F209" t="inlineStr"/>
       <c r="G209" s="6" t="n">
         <v>60346</v>
       </c>
@@ -11884,8 +11705,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E210" t="inlineStr"/>
-      <c r="F210" t="inlineStr"/>
       <c r="G210" s="6" t="n">
         <v>52676</v>
       </c>
@@ -11933,8 +11752,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E211" t="inlineStr"/>
-      <c r="F211" t="inlineStr"/>
       <c r="G211" s="6" t="n">
         <v>53397</v>
       </c>
@@ -11982,8 +11799,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E212" t="inlineStr"/>
-      <c r="F212" t="inlineStr"/>
       <c r="G212" s="6" t="n">
         <v>67853</v>
       </c>
@@ -12031,8 +11846,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E213" t="inlineStr"/>
-      <c r="F213" t="inlineStr"/>
       <c r="G213" s="6" t="n">
         <v>61371</v>
       </c>
@@ -12080,8 +11893,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E214" t="inlineStr"/>
-      <c r="F214" t="inlineStr"/>
       <c r="G214" s="6" t="n">
         <v>69157</v>
       </c>
@@ -12129,8 +11940,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E215" t="inlineStr"/>
-      <c r="F215" t="inlineStr"/>
       <c r="G215" s="6" t="n">
         <v>61909</v>
       </c>
@@ -12178,8 +11987,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E216" t="inlineStr"/>
-      <c r="F216" t="inlineStr"/>
       <c r="G216" s="6" t="n">
         <v>70220</v>
       </c>
@@ -12227,8 +12034,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E217" t="inlineStr"/>
-      <c r="F217" t="inlineStr"/>
       <c r="G217" s="6" t="n">
         <v>71273</v>
       </c>
@@ -12276,8 +12081,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E218" t="inlineStr"/>
-      <c r="F218" t="inlineStr"/>
       <c r="G218" s="6" t="n">
         <v>16373</v>
       </c>
@@ -12325,8 +12128,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E219" t="inlineStr"/>
-      <c r="F219" t="inlineStr"/>
       <c r="G219" s="6" t="n">
         <v>19173</v>
       </c>
@@ -12374,8 +12175,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr"/>
-      <c r="F220" t="inlineStr"/>
       <c r="G220" s="6" t="n">
         <v>24869</v>
       </c>
@@ -12423,8 +12222,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E221" t="inlineStr"/>
-      <c r="F221" t="inlineStr"/>
       <c r="G221" s="6" t="n">
         <v>30450</v>
       </c>
@@ -12472,8 +12269,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E222" t="inlineStr"/>
-      <c r="F222" t="inlineStr"/>
       <c r="G222" s="6" t="n">
         <v>29342</v>
       </c>
@@ -12521,8 +12316,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr"/>
-      <c r="F223" t="inlineStr"/>
       <c r="G223" s="6" t="n">
         <v>35927</v>
       </c>
@@ -12570,8 +12363,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr"/>
-      <c r="F224" t="inlineStr"/>
       <c r="G224" s="6" t="n">
         <v>39577</v>
       </c>
@@ -12619,8 +12410,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E225" t="inlineStr"/>
-      <c r="F225" t="inlineStr"/>
       <c r="G225" s="6" t="n">
         <v>46038</v>
       </c>
@@ -12668,8 +12457,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E226" t="inlineStr"/>
-      <c r="F226" t="inlineStr"/>
       <c r="G226" s="6" t="n">
         <v>42389</v>
       </c>
@@ -12717,8 +12504,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E227" t="inlineStr"/>
-      <c r="F227" t="inlineStr"/>
       <c r="G227" s="6" t="n">
         <v>50476</v>
       </c>
@@ -12766,8 +12551,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E228" t="inlineStr"/>
-      <c r="F228" t="inlineStr"/>
       <c r="G228" s="6" t="n">
         <v>62169</v>
       </c>
@@ -12815,8 +12598,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E229" t="inlineStr"/>
-      <c r="F229" t="inlineStr"/>
       <c r="G229" s="6" t="n">
         <v>54318</v>
       </c>
@@ -12864,8 +12645,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E230" t="inlineStr"/>
-      <c r="F230" t="inlineStr"/>
       <c r="G230" s="6" t="n">
         <v>50013</v>
       </c>
@@ -12913,8 +12692,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E231" t="inlineStr"/>
-      <c r="F231" t="inlineStr"/>
       <c r="G231" s="6" t="n">
         <v>66756</v>
       </c>
@@ -12962,8 +12739,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E232" t="inlineStr"/>
-      <c r="F232" t="inlineStr"/>
       <c r="G232" s="6" t="n">
         <v>62080</v>
       </c>
@@ -13011,8 +12786,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E233" t="inlineStr"/>
-      <c r="F233" t="inlineStr"/>
       <c r="G233" s="6" t="n">
         <v>58987</v>
       </c>
@@ -13060,8 +12833,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E234" t="inlineStr"/>
-      <c r="F234" t="inlineStr"/>
       <c r="G234" s="6" t="n">
         <v>51073</v>
       </c>
@@ -13109,8 +12880,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E235" t="inlineStr"/>
-      <c r="F235" t="inlineStr"/>
       <c r="G235" s="6" t="n">
         <v>53189</v>
       </c>
@@ -13158,8 +12927,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr"/>
-      <c r="F236" t="inlineStr"/>
       <c r="G236" s="6" t="n">
         <v>67032</v>
       </c>
@@ -13207,8 +12974,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E237" t="inlineStr"/>
-      <c r="F237" t="inlineStr"/>
       <c r="G237" s="6" t="n">
         <v>63178</v>
       </c>
@@ -13256,8 +13021,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E238" t="inlineStr"/>
-      <c r="F238" t="inlineStr"/>
       <c r="G238" s="6" t="n">
         <v>54140</v>
       </c>
@@ -13305,8 +13068,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E239" t="inlineStr"/>
-      <c r="F239" t="inlineStr"/>
       <c r="G239" s="6" t="n">
         <v>71795</v>
       </c>
@@ -13354,8 +13115,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E240" t="inlineStr"/>
-      <c r="F240" t="inlineStr"/>
       <c r="G240" s="6" t="n">
         <v>69596</v>
       </c>
@@ -13403,8 +13162,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E241" t="inlineStr"/>
-      <c r="F241" t="inlineStr"/>
       <c r="G241" s="6" t="n">
         <v>73847</v>
       </c>
@@ -13452,8 +13209,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E242" t="inlineStr"/>
-      <c r="F242" t="inlineStr"/>
       <c r="G242" s="6" t="n">
         <v>84767</v>
       </c>
@@ -13501,8 +13256,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E243" t="inlineStr"/>
-      <c r="F243" t="inlineStr"/>
       <c r="G243" s="6" t="n">
         <v>70527</v>
       </c>
@@ -13550,8 +13303,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr"/>
-      <c r="F244" t="inlineStr"/>
       <c r="G244" s="6" t="n">
         <v>71362</v>
       </c>
@@ -13599,8 +13350,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E245" t="inlineStr"/>
-      <c r="F245" t="inlineStr"/>
       <c r="G245" s="6" t="n">
         <v>77589</v>
       </c>
@@ -13648,8 +13397,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E246" t="inlineStr"/>
-      <c r="F246" t="inlineStr"/>
       <c r="G246" s="6" t="n">
         <v>89366</v>
       </c>
@@ -13697,8 +13444,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E247" t="inlineStr"/>
-      <c r="F247" t="inlineStr"/>
       <c r="G247" s="6" t="n">
         <v>93443</v>
       </c>
@@ -13746,8 +13491,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E248" t="inlineStr"/>
-      <c r="F248" t="inlineStr"/>
       <c r="G248" s="6" t="n">
         <v>100937</v>
       </c>
@@ -13795,8 +13538,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E249" t="inlineStr"/>
-      <c r="F249" t="inlineStr"/>
       <c r="G249" s="6" t="n">
         <v>101454</v>
       </c>
@@ -16316,19 +16057,25 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E295" t="inlineStr"/>
-      <c r="F295" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>price list 2019 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G295" s="6" t="n">
         <v>1205</v>
       </c>
       <c r="H295" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I295" s="3" t="n">
-        <v>1550</v>
+        <v>2500</v>
       </c>
       <c r="J295">
         <f>IF(I295&gt;0,CEILING(I295*(1-Policy!$B$13/100),IF(I295&lt;10000,50,100)),"")</f>
@@ -16369,11 +16116,11 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>1800</v>
+        <v>2200</v>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>product_list:market</t>
+          <t>price list 2019 (Price List India 2022-23.pdf)</t>
         </is>
       </c>
       <c r="G296" t="n">
@@ -16383,7 +16130,7 @@
         <v>0</v>
       </c>
       <c r="I296" s="3" t="n">
-        <v>1800</v>
+        <v>2200</v>
       </c>
       <c r="J296">
         <f>IF(I296&gt;0,CEILING(I296*(1-Policy!$B$13/100),IF(I296&lt;10000,50,100)),"")</f>
@@ -16533,8 +16280,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E299" t="inlineStr"/>
-      <c r="F299" t="inlineStr"/>
       <c r="G299" s="6" t="n">
         <v>5461</v>
       </c>
@@ -16582,8 +16327,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E300" t="inlineStr"/>
-      <c r="F300" t="inlineStr"/>
       <c r="G300" s="6" t="n">
         <v>5461</v>
       </c>
@@ -20689,11 +20432,11 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>25000</v>
+        <v>15500</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>confirmed by Paresh 24-09-2026</t>
+          <t>Paresh 25-09-2026, from WR costing sheets</t>
         </is>
       </c>
       <c r="G62" t="n">
@@ -23755,8 +23498,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" s="6" t="n">
         <v>1200</v>
       </c>
@@ -23804,8 +23545,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" s="6" t="n">
         <v>1200</v>
       </c>
@@ -23853,8 +23592,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" s="6" t="n">
         <v>2200</v>
       </c>
@@ -23902,8 +23639,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" s="6" t="n">
         <v>1500</v>
       </c>
@@ -23951,8 +23686,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" s="6" t="n">
         <v>2600</v>
       </c>
@@ -24000,8 +23733,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" s="6" t="n">
         <v>1800</v>
       </c>
@@ -24049,8 +23780,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" s="6" t="n">
         <v>450</v>
       </c>
@@ -24098,8 +23827,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" s="6" t="n">
         <v>2400</v>
       </c>
@@ -24147,8 +23874,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" s="6" t="n">
         <v>900</v>
       </c>
@@ -24196,8 +23921,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" s="6" t="n">
         <v>250</v>
       </c>
@@ -24245,8 +23968,6 @@
           <t>on request</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" s="6" t="n">
         <v>0</v>
       </c>
@@ -24294,8 +24015,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" s="6" t="n">
         <v>350</v>
       </c>
@@ -24343,8 +24062,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" s="6" t="n">
         <v>600</v>
       </c>
@@ -24392,8 +24109,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" s="6" t="n">
         <v>900</v>
       </c>
@@ -24441,8 +24156,6 @@
           <t>on request</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" s="6" t="n">
         <v>0</v>
       </c>
@@ -24490,8 +24203,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" s="6" t="n">
         <v>6500</v>
       </c>
@@ -24539,8 +24250,6 @@
           <t>on request</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" s="6" t="n">
         <v>0</v>
       </c>
@@ -24713,7 +24422,6 @@
       <c r="L2" t="n">
         <v>21</v>
       </c>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -24764,7 +24472,6 @@
       <c r="L3" t="n">
         <v>21</v>
       </c>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -24815,7 +24522,6 @@
       <c r="L4" t="n">
         <v>21</v>
       </c>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -24866,7 +24572,6 @@
       <c r="L5" t="n">
         <v>21</v>
       </c>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -24917,7 +24622,6 @@
       <c r="L6" t="n">
         <v>21</v>
       </c>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -24968,7 +24672,6 @@
       <c r="L7" t="n">
         <v>21</v>
       </c>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -25019,7 +24722,6 @@
       <c r="L8" t="n">
         <v>21</v>
       </c>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -25070,7 +24772,6 @@
       <c r="L9" t="n">
         <v>21</v>
       </c>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -25121,7 +24822,6 @@
       <c r="L10" t="n">
         <v>21</v>
       </c>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -25172,7 +24872,6 @@
       <c r="L11" t="n">
         <v>21</v>
       </c>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -25223,7 +24922,6 @@
       <c r="L12" t="n">
         <v>21</v>
       </c>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -25274,7 +24972,6 @@
       <c r="L13" t="n">
         <v>21</v>
       </c>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -25325,7 +25022,6 @@
       <c r="L14" t="n">
         <v>21</v>
       </c>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -25376,7 +25072,6 @@
       <c r="L15" t="n">
         <v>21</v>
       </c>
-      <c r="M15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M15"/>
@@ -33640,9 +33335,6 @@
       <c r="D94" t="n">
         <v>1150</v>
       </c>
-      <c r="E94" t="inlineStr"/>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" s="3" t="n">
         <v>4</v>
       </c>
@@ -33720,9 +33412,6 @@
       <c r="D95" t="n">
         <v>1750</v>
       </c>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
-      <c r="G95" t="inlineStr"/>
       <c r="H95" s="3" t="n">
         <v>4</v>
       </c>
@@ -33800,9 +33489,6 @@
       <c r="D96" t="n">
         <v>2200</v>
       </c>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
       <c r="H96" s="3" t="n">
         <v>4</v>
       </c>
@@ -33880,9 +33566,6 @@
       <c r="D97" t="n">
         <v>2200</v>
       </c>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
       <c r="H97" s="3" t="n">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
Name fix, catalogue photos, delete buttons, file attach on approval
</commit_message>
<xml_diff>
--- a/pricing/ImpactCal_Pricelist_2026-09.xlsx
+++ b/pricing/ImpactCal_Pricelist_2026-09.xlsx
@@ -475,6 +475,8 @@
           <t>ADONI TECH — ImpactCal global price list &amp; costing</t>
         </is>
       </c>
+      <c r="B1" t="inlineStr"/>
+      <c r="C1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -487,14 +489,20 @@
           <t>2026-09-24</t>
         </is>
       </c>
-    </row>
-    <row r="3"/>
+      <c r="C2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+    </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>PRICING POLICY (agreed 23-24 Sep 2026)</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -507,6 +515,7 @@
           <t>Highest price found in any of the 8 uploaded price lists is taken as-is (list price).</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -519,6 +528,7 @@
           <t>Cost model per series (price ~ k · Fs^a · stroke^b fitted on your own prices; median error 6 % crane, 9 % industrial) + negotiation margin below</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -531,6 +541,7 @@
           <t>Moulding cost + hardware + mould cost amortised, + margin over cost (parameters below; Rubber mounts sheet recalculates live)</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -543,6 +554,7 @@
           <t>nearest ₹50 below ₹10,000, nearest ₹100 above (always up)</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -555,8 +567,12 @@
           <t>list ÷ live INR/USD rate × (1 + export uplift); recomputed at quotation time; column here is indicative</t>
         </is>
       </c>
-    </row>
-    <row r="10"/>
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+    </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -795,6 +811,7 @@
           <t>8 / 4 / 1</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1027,6 +1044,8 @@
           <t>blue = estimated value</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1366,11 +1385,11 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1100</v>
+        <v>980</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>price list 2019 (Price List India 2022-23.pdf)</t>
+          <t>product_list:market</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -1380,7 +1399,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="J6">
         <f>IF(I6&gt;0,CEILING(I6*(1-Policy!$B$13/100),IF(I6&lt;10000,50,100)),"")</f>
@@ -1640,6 +1659,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" s="6" t="n">
         <v>3669</v>
       </c>
@@ -2509,25 +2530,19 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>11000</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
-        </is>
-      </c>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" s="6" t="n">
         <v>13156</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>11000</v>
+        <v>16500</v>
       </c>
       <c r="J27">
         <f>IF(I27&gt;0,CEILING(I27*(1-Policy!$B$13/100),IF(I27&lt;10000,50,100)),"")</f>
@@ -2564,25 +2579,19 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>12500</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
-        </is>
-      </c>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" s="6" t="n">
         <v>15556</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>12500</v>
+        <v>19500</v>
       </c>
       <c r="J28">
         <f>IF(I28&gt;0,CEILING(I28*(1-Policy!$B$13/100),IF(I28&lt;10000,50,100)),"")</f>
@@ -2622,6 +2631,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" s="6" t="n">
         <v>22637</v>
       </c>
@@ -2669,6 +2680,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" s="6" t="n">
         <v>22711</v>
       </c>
@@ -2716,6 +2729,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" s="6" t="n">
         <v>30472</v>
       </c>
@@ -2763,6 +2778,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" s="6" t="n">
         <v>32765</v>
       </c>
@@ -2810,6 +2827,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" s="6" t="n">
         <v>35158</v>
       </c>
@@ -2857,6 +2876,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" s="6" t="n">
         <v>4638</v>
       </c>
@@ -2904,6 +2925,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" s="6" t="n">
         <v>4638</v>
       </c>
@@ -2951,6 +2974,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" s="6" t="n">
         <v>6578</v>
       </c>
@@ -3053,6 +3078,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" s="6" t="n">
         <v>8783</v>
       </c>
@@ -3100,6 +3127,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" s="6" t="n">
         <v>12227</v>
       </c>
@@ -3147,6 +3176,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" s="6" t="n">
         <v>14740</v>
       </c>
@@ -3194,6 +3225,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" s="6" t="n">
         <v>16533</v>
       </c>
@@ -3242,11 +3275,11 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1400</v>
+        <v>1300</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>price list 2019 (Price List India 2022-23.pdf)</t>
+          <t>product_list:b2b</t>
         </is>
       </c>
       <c r="G42" t="n">
@@ -3256,7 +3289,7 @@
         <v>0</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>1400</v>
+        <v>1300</v>
       </c>
       <c r="J42">
         <f>IF(I42&gt;0,CEILING(I42*(1-Policy!$B$13/100),IF(I42&lt;10000,50,100)),"")</f>
@@ -3297,11 +3330,11 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>2400</v>
+        <v>2200</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>price list 2019 (Price List India 2022-23.pdf)</t>
+          <t>product_list:market</t>
         </is>
       </c>
       <c r="G43" t="n">
@@ -3311,7 +3344,7 @@
         <v>0</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>2400</v>
+        <v>2200</v>
       </c>
       <c r="J43">
         <f>IF(I43&gt;0,CEILING(I43*(1-Policy!$B$13/100),IF(I43&lt;10000,50,100)),"")</f>
@@ -3461,6 +3494,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" s="6" t="n">
         <v>4235</v>
       </c>
@@ -4110,25 +4145,19 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="E58" t="n">
-        <v>8500</v>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
-        </is>
-      </c>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" s="6" t="n">
         <v>7701</v>
       </c>
       <c r="H58" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>8500</v>
+        <v>9650</v>
       </c>
       <c r="J58">
         <f>IF(I58&gt;0,CEILING(I58*(1-Policy!$B$13/100),IF(I58&lt;10000,50,100)),"")</f>
@@ -4220,25 +4249,19 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="E60" t="n">
-        <v>11800</v>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
-        </is>
-      </c>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" s="6" t="n">
         <v>9296</v>
       </c>
       <c r="H60" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>11800</v>
+        <v>11700</v>
       </c>
       <c r="J60">
         <f>IF(I60&gt;0,CEILING(I60*(1-Policy!$B$13/100),IF(I60&lt;10000,50,100)),"")</f>
@@ -4275,25 +4298,19 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="E61" t="n">
-        <v>12000</v>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
-        </is>
-      </c>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
       <c r="G61" s="6" t="n">
         <v>10378</v>
       </c>
       <c r="H61" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I61" s="3" t="n">
-        <v>12000</v>
+        <v>13000</v>
       </c>
       <c r="J61">
         <f>IF(I61&gt;0,CEILING(I61*(1-Policy!$B$13/100),IF(I61&lt;10000,50,100)),"")</f>
@@ -4330,25 +4347,19 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="E62" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
-        </is>
-      </c>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
       <c r="G62" s="6" t="n">
         <v>14212</v>
       </c>
       <c r="H62" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>15000</v>
+        <v>17800</v>
       </c>
       <c r="J62">
         <f>IF(I62&gt;0,CEILING(I62*(1-Policy!$B$13/100),IF(I62&lt;10000,50,100)),"")</f>
@@ -4385,25 +4396,19 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="E63" t="n">
-        <v>17500</v>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
-        </is>
-      </c>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
       <c r="G63" s="6" t="n">
         <v>16805</v>
       </c>
       <c r="H63" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>17500</v>
+        <v>21100</v>
       </c>
       <c r="J63">
         <f>IF(I63&gt;0,CEILING(I63*(1-Policy!$B$13/100),IF(I63&lt;10000,50,100)),"")</f>
@@ -4498,6 +4503,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
       <c r="G65" s="6" t="n">
         <v>40131</v>
       </c>
@@ -4542,25 +4549,19 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="E66" t="n">
-        <v>44000</v>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
-        </is>
-      </c>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" s="6" t="n">
         <v>32918</v>
       </c>
       <c r="H66" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>44000</v>
+        <v>41200</v>
       </c>
       <c r="J66">
         <f>IF(I66&gt;0,CEILING(I66*(1-Policy!$B$13/100),IF(I66&lt;10000,50,100)),"")</f>
@@ -4597,25 +4598,19 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="E67" t="n">
-        <v>50000</v>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
-        </is>
-      </c>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" s="6" t="n">
         <v>35395</v>
       </c>
       <c r="H67" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I67" s="3" t="n">
-        <v>50000</v>
+        <v>44300</v>
       </c>
       <c r="J67">
         <f>IF(I67&gt;0,CEILING(I67*(1-Policy!$B$13/100),IF(I67&lt;10000,50,100)),"")</f>
@@ -4652,25 +4647,19 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="E68" t="n">
-        <v>55000</v>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
-        </is>
-      </c>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
       <c r="G68" s="6" t="n">
         <v>37981</v>
       </c>
       <c r="H68" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>55000</v>
+        <v>47500</v>
       </c>
       <c r="J68">
         <f>IF(I68&gt;0,CEILING(I68*(1-Policy!$B$13/100),IF(I68&lt;10000,50,100)),"")</f>
@@ -4930,6 +4919,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
       <c r="G73" s="6" t="n">
         <v>20689</v>
       </c>
@@ -5362,6 +5353,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
       <c r="G81" s="6" t="n">
         <v>26890</v>
       </c>
@@ -5904,6 +5897,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
       <c r="G91" s="6" t="n">
         <v>52785</v>
       </c>
@@ -5951,6 +5946,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
       <c r="G92" s="6" t="n">
         <v>60795</v>
       </c>
@@ -5998,6 +5995,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
       <c r="G93" s="6" t="n">
         <v>68832</v>
       </c>
@@ -6265,6 +6264,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" s="6" t="n">
         <v>58913</v>
       </c>
@@ -6312,6 +6313,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
       <c r="G99" s="6" t="n">
         <v>69090</v>
       </c>
@@ -6524,6 +6527,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
       <c r="G103" s="6" t="n">
         <v>70653</v>
       </c>
@@ -6736,6 +6741,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
       <c r="G107" s="6" t="n">
         <v>81211</v>
       </c>
@@ -6948,6 +6955,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
       <c r="G111" s="6" t="n">
         <v>73543</v>
       </c>
@@ -7050,6 +7059,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
       <c r="G113" s="6" t="n">
         <v>85653</v>
       </c>
@@ -7482,6 +7493,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
       <c r="G121" s="6" t="n">
         <v>89371</v>
       </c>
@@ -7529,6 +7542,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
       <c r="G122" s="6" t="n">
         <v>80189</v>
       </c>
@@ -7686,6 +7701,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
       <c r="G125" s="6" t="n">
         <v>81294</v>
       </c>
@@ -7788,6 +7805,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
       <c r="G127" s="6" t="n">
         <v>94259</v>
       </c>
@@ -7890,6 +7909,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
       <c r="G129" s="6" t="n">
         <v>80100</v>
       </c>
@@ -7937,6 +7958,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
       <c r="G130" s="6" t="n">
         <v>79673</v>
       </c>
@@ -7984,6 +8007,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
       <c r="G131" s="6" t="n">
         <v>99666</v>
       </c>
@@ -8031,6 +8056,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
       <c r="G132" s="6" t="n">
         <v>106423</v>
       </c>
@@ -8078,6 +8105,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
       <c r="G133" s="6" t="n">
         <v>112858</v>
       </c>
@@ -8180,6 +8209,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
       <c r="G135" s="6" t="n">
         <v>29935</v>
       </c>
@@ -8227,6 +8258,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
       <c r="G136" s="6" t="n">
         <v>31513</v>
       </c>
@@ -8274,6 +8307,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
       <c r="G137" s="6" t="n">
         <v>42694</v>
       </c>
@@ -8321,6 +8356,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
       <c r="G138" s="6" t="n">
         <v>49521</v>
       </c>
@@ -8368,6 +8405,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
       <c r="G139" s="6" t="n">
         <v>45237</v>
       </c>
@@ -8415,6 +8454,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
       <c r="G140" s="6" t="n">
         <v>55448</v>
       </c>
@@ -8462,6 +8503,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
       <c r="G141" s="6" t="n">
         <v>15625</v>
       </c>
@@ -8509,6 +8552,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
       <c r="G142" s="6" t="n">
         <v>17980</v>
       </c>
@@ -8556,6 +8601,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
       <c r="G143" s="6" t="n">
         <v>19750</v>
       </c>
@@ -8603,6 +8650,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
       <c r="G144" s="6" t="n">
         <v>27713</v>
       </c>
@@ -8650,6 +8699,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
       <c r="G145" s="6" t="n">
         <v>21214</v>
       </c>
@@ -8697,6 +8748,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
       <c r="G146" s="6" t="n">
         <v>32461</v>
       </c>
@@ -8744,6 +8797,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
       <c r="G147" s="6" t="n">
         <v>30749</v>
       </c>
@@ -8791,6 +8846,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
       <c r="G148" s="6" t="n">
         <v>22335</v>
       </c>
@@ -8838,6 +8895,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
       <c r="G149" s="6" t="n">
         <v>35819</v>
       </c>
@@ -8885,6 +8944,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
       <c r="G150" s="6" t="n">
         <v>27425</v>
       </c>
@@ -8932,6 +8993,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
       <c r="G151" s="6" t="n">
         <v>23369</v>
       </c>
@@ -8979,6 +9042,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr"/>
       <c r="G152" s="6" t="n">
         <v>23976</v>
       </c>
@@ -9026,6 +9091,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr"/>
       <c r="G153" s="6" t="n">
         <v>29404</v>
       </c>
@@ -9073,6 +9140,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr"/>
       <c r="G154" s="6" t="n">
         <v>24434</v>
       </c>
@@ -9120,6 +9189,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr"/>
       <c r="G155" s="6" t="n">
         <v>34635</v>
       </c>
@@ -9167,6 +9238,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E156" t="inlineStr"/>
+      <c r="F156" t="inlineStr"/>
       <c r="G156" s="6" t="n">
         <v>24670</v>
       </c>
@@ -9214,6 +9287,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr"/>
       <c r="G157" s="6" t="n">
         <v>38300</v>
       </c>
@@ -9261,6 +9336,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E158" t="inlineStr"/>
+      <c r="F158" t="inlineStr"/>
       <c r="G158" s="6" t="n">
         <v>24867</v>
       </c>
@@ -9308,6 +9385,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr"/>
       <c r="G159" s="6" t="n">
         <v>31172</v>
       </c>
@@ -9355,6 +9434,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr"/>
       <c r="G160" s="6" t="n">
         <v>25070</v>
       </c>
@@ -9402,6 +9483,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E161" t="inlineStr"/>
+      <c r="F161" t="inlineStr"/>
       <c r="G161" s="6" t="n">
         <v>42121</v>
       </c>
@@ -9449,6 +9532,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr"/>
       <c r="G162" s="6" t="n">
         <v>25112</v>
       </c>
@@ -9496,6 +9581,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr"/>
       <c r="G163" s="6" t="n">
         <v>32430</v>
       </c>
@@ -9543,6 +9630,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr"/>
       <c r="G164" s="6" t="n">
         <v>37139</v>
       </c>
@@ -9590,6 +9679,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr"/>
       <c r="G165" s="6" t="n">
         <v>25264</v>
       </c>
@@ -9637,6 +9728,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr"/>
       <c r="G166" s="6" t="n">
         <v>33063</v>
       </c>
@@ -9684,6 +9777,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E167" t="inlineStr"/>
+      <c r="F167" t="inlineStr"/>
       <c r="G167" s="6" t="n">
         <v>42077</v>
       </c>
@@ -9731,6 +9826,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E168" t="inlineStr"/>
+      <c r="F168" t="inlineStr"/>
       <c r="G168" s="6" t="n">
         <v>33717</v>
       </c>
@@ -9778,6 +9875,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E169" t="inlineStr"/>
+      <c r="F169" t="inlineStr"/>
       <c r="G169" s="6" t="n">
         <v>38513</v>
       </c>
@@ -9825,6 +9924,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E170" t="inlineStr"/>
+      <c r="F170" t="inlineStr"/>
       <c r="G170" s="6" t="n">
         <v>46129</v>
       </c>
@@ -9872,6 +9973,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr"/>
       <c r="G171" s="6" t="n">
         <v>34304</v>
       </c>
@@ -9919,6 +10022,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E172" t="inlineStr"/>
+      <c r="F172" t="inlineStr"/>
       <c r="G172" s="6" t="n">
         <v>39761</v>
       </c>
@@ -9966,6 +10071,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E173" t="inlineStr"/>
+      <c r="F173" t="inlineStr"/>
       <c r="G173" s="6" t="n">
         <v>44687</v>
       </c>
@@ -10013,6 +10120,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E174" t="inlineStr"/>
+      <c r="F174" t="inlineStr"/>
       <c r="G174" s="6" t="n">
         <v>34832</v>
       </c>
@@ -10060,6 +10169,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E175" t="inlineStr"/>
+      <c r="F175" t="inlineStr"/>
       <c r="G175" s="6" t="n">
         <v>35928</v>
       </c>
@@ -10107,6 +10218,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E176" t="inlineStr"/>
+      <c r="F176" t="inlineStr"/>
       <c r="G176" s="6" t="n">
         <v>46027</v>
       </c>
@@ -10154,6 +10267,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E177" t="inlineStr"/>
+      <c r="F177" t="inlineStr"/>
       <c r="G177" s="6" t="n">
         <v>49530</v>
       </c>
@@ -10201,6 +10316,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr"/>
       <c r="G178" s="6" t="n">
         <v>42595</v>
       </c>
@@ -10248,6 +10365,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E179" t="inlineStr"/>
+      <c r="F179" t="inlineStr"/>
       <c r="G179" s="6" t="n">
         <v>36962</v>
       </c>
@@ -10295,6 +10414,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E180" t="inlineStr"/>
+      <c r="F180" t="inlineStr"/>
       <c r="G180" s="6" t="n">
         <v>43498</v>
       </c>
@@ -10342,6 +10463,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr"/>
       <c r="G181" s="6" t="n">
         <v>35830</v>
       </c>
@@ -10389,6 +10512,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr"/>
       <c r="G182" s="6" t="n">
         <v>47326</v>
       </c>
@@ -10436,6 +10561,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr"/>
       <c r="G183" s="6" t="n">
         <v>52098</v>
       </c>
@@ -10483,6 +10610,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E184" t="inlineStr"/>
+      <c r="F184" t="inlineStr"/>
       <c r="G184" s="6" t="n">
         <v>44353</v>
       </c>
@@ -10530,6 +10659,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E185" t="inlineStr"/>
+      <c r="F185" t="inlineStr"/>
       <c r="G185" s="6" t="n">
         <v>45164</v>
       </c>
@@ -10577,6 +10708,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E186" t="inlineStr"/>
+      <c r="F186" t="inlineStr"/>
       <c r="G186" s="6" t="n">
         <v>49586</v>
       </c>
@@ -10624,6 +10757,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E187" t="inlineStr"/>
+      <c r="F187" t="inlineStr"/>
       <c r="G187" s="6" t="n">
         <v>54439</v>
       </c>
@@ -10671,6 +10806,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E188" t="inlineStr"/>
+      <c r="F188" t="inlineStr"/>
       <c r="G188" s="6" t="n">
         <v>46646</v>
       </c>
@@ -10718,6 +10855,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E189" t="inlineStr"/>
+      <c r="F189" t="inlineStr"/>
       <c r="G189" s="6" t="n">
         <v>41784</v>
       </c>
@@ -10765,6 +10904,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E190" t="inlineStr"/>
+      <c r="F190" t="inlineStr"/>
       <c r="G190" s="6" t="n">
         <v>40599</v>
       </c>
@@ -10812,6 +10953,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E191" t="inlineStr"/>
+      <c r="F191" t="inlineStr"/>
       <c r="G191" s="6" t="n">
         <v>41080</v>
       </c>
@@ -10859,6 +11002,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E192" t="inlineStr"/>
+      <c r="F192" t="inlineStr"/>
       <c r="G192" s="6" t="n">
         <v>48023</v>
       </c>
@@ -10906,6 +11051,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E193" t="inlineStr"/>
+      <c r="F193" t="inlineStr"/>
       <c r="G193" s="6" t="n">
         <v>53650</v>
       </c>
@@ -10953,6 +11100,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E194" t="inlineStr"/>
+      <c r="F194" t="inlineStr"/>
       <c r="G194" s="6" t="n">
         <v>58216</v>
       </c>
@@ -11000,6 +11149,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E195" t="inlineStr"/>
+      <c r="F195" t="inlineStr"/>
       <c r="G195" s="6" t="n">
         <v>41168</v>
       </c>
@@ -11047,6 +11198,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E196" t="inlineStr"/>
+      <c r="F196" t="inlineStr"/>
       <c r="G196" s="6" t="n">
         <v>49268</v>
       </c>
@@ -11094,6 +11247,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E197" t="inlineStr"/>
+      <c r="F197" t="inlineStr"/>
       <c r="G197" s="6" t="n">
         <v>55239</v>
       </c>
@@ -11141,6 +11296,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E198" t="inlineStr"/>
+      <c r="F198" t="inlineStr"/>
       <c r="G198" s="6" t="n">
         <v>50893</v>
       </c>
@@ -11188,6 +11345,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E199" t="inlineStr"/>
+      <c r="F199" t="inlineStr"/>
       <c r="G199" s="6" t="n">
         <v>61426</v>
       </c>
@@ -11235,6 +11394,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr"/>
       <c r="G200" s="6" t="n">
         <v>56693</v>
       </c>
@@ -11282,6 +11443,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E201" t="inlineStr"/>
+      <c r="F201" t="inlineStr"/>
       <c r="G201" s="6" t="n">
         <v>51435</v>
       </c>
@@ -11329,6 +11492,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E202" t="inlineStr"/>
+      <c r="F202" t="inlineStr"/>
       <c r="G202" s="6" t="n">
         <v>58064</v>
       </c>
@@ -11376,6 +11541,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E203" t="inlineStr"/>
+      <c r="F203" t="inlineStr"/>
       <c r="G203" s="6" t="n">
         <v>51967</v>
       </c>
@@ -11423,6 +11590,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E204" t="inlineStr"/>
+      <c r="F204" t="inlineStr"/>
       <c r="G204" s="6" t="n">
         <v>64157</v>
       </c>
@@ -11470,6 +11639,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E205" t="inlineStr"/>
+      <c r="F205" t="inlineStr"/>
       <c r="G205" s="6" t="n">
         <v>52150</v>
       </c>
@@ -11517,6 +11688,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E206" t="inlineStr"/>
+      <c r="F206" t="inlineStr"/>
       <c r="G206" s="6" t="n">
         <v>59346</v>
       </c>
@@ -11564,6 +11737,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E207" t="inlineStr"/>
+      <c r="F207" t="inlineStr"/>
       <c r="G207" s="6" t="n">
         <v>52495</v>
       </c>
@@ -11611,6 +11786,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E208" t="inlineStr"/>
+      <c r="F208" t="inlineStr"/>
       <c r="G208" s="6" t="n">
         <v>66481</v>
       </c>
@@ -11658,6 +11835,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E209" t="inlineStr"/>
+      <c r="F209" t="inlineStr"/>
       <c r="G209" s="6" t="n">
         <v>60346</v>
       </c>
@@ -11705,6 +11884,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E210" t="inlineStr"/>
+      <c r="F210" t="inlineStr"/>
       <c r="G210" s="6" t="n">
         <v>52676</v>
       </c>
@@ -11752,6 +11933,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E211" t="inlineStr"/>
+      <c r="F211" t="inlineStr"/>
       <c r="G211" s="6" t="n">
         <v>53397</v>
       </c>
@@ -11799,6 +11982,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E212" t="inlineStr"/>
+      <c r="F212" t="inlineStr"/>
       <c r="G212" s="6" t="n">
         <v>67853</v>
       </c>
@@ -11846,6 +12031,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E213" t="inlineStr"/>
+      <c r="F213" t="inlineStr"/>
       <c r="G213" s="6" t="n">
         <v>61371</v>
       </c>
@@ -11893,6 +12080,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E214" t="inlineStr"/>
+      <c r="F214" t="inlineStr"/>
       <c r="G214" s="6" t="n">
         <v>69157</v>
       </c>
@@ -11940,6 +12129,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E215" t="inlineStr"/>
+      <c r="F215" t="inlineStr"/>
       <c r="G215" s="6" t="n">
         <v>61909</v>
       </c>
@@ -11987,6 +12178,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E216" t="inlineStr"/>
+      <c r="F216" t="inlineStr"/>
       <c r="G216" s="6" t="n">
         <v>70220</v>
       </c>
@@ -12034,6 +12227,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E217" t="inlineStr"/>
+      <c r="F217" t="inlineStr"/>
       <c r="G217" s="6" t="n">
         <v>71273</v>
       </c>
@@ -12081,6 +12276,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E218" t="inlineStr"/>
+      <c r="F218" t="inlineStr"/>
       <c r="G218" s="6" t="n">
         <v>16373</v>
       </c>
@@ -12128,6 +12325,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E219" t="inlineStr"/>
+      <c r="F219" t="inlineStr"/>
       <c r="G219" s="6" t="n">
         <v>19173</v>
       </c>
@@ -12175,6 +12374,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E220" t="inlineStr"/>
+      <c r="F220" t="inlineStr"/>
       <c r="G220" s="6" t="n">
         <v>24869</v>
       </c>
@@ -12222,6 +12423,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E221" t="inlineStr"/>
+      <c r="F221" t="inlineStr"/>
       <c r="G221" s="6" t="n">
         <v>30450</v>
       </c>
@@ -12269,6 +12472,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E222" t="inlineStr"/>
+      <c r="F222" t="inlineStr"/>
       <c r="G222" s="6" t="n">
         <v>29342</v>
       </c>
@@ -12316,6 +12521,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E223" t="inlineStr"/>
+      <c r="F223" t="inlineStr"/>
       <c r="G223" s="6" t="n">
         <v>35927</v>
       </c>
@@ -12363,6 +12570,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E224" t="inlineStr"/>
+      <c r="F224" t="inlineStr"/>
       <c r="G224" s="6" t="n">
         <v>39577</v>
       </c>
@@ -12410,6 +12619,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E225" t="inlineStr"/>
+      <c r="F225" t="inlineStr"/>
       <c r="G225" s="6" t="n">
         <v>46038</v>
       </c>
@@ -12457,6 +12668,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E226" t="inlineStr"/>
+      <c r="F226" t="inlineStr"/>
       <c r="G226" s="6" t="n">
         <v>42389</v>
       </c>
@@ -12504,6 +12717,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E227" t="inlineStr"/>
+      <c r="F227" t="inlineStr"/>
       <c r="G227" s="6" t="n">
         <v>50476</v>
       </c>
@@ -12551,6 +12766,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E228" t="inlineStr"/>
+      <c r="F228" t="inlineStr"/>
       <c r="G228" s="6" t="n">
         <v>62169</v>
       </c>
@@ -12598,6 +12815,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E229" t="inlineStr"/>
+      <c r="F229" t="inlineStr"/>
       <c r="G229" s="6" t="n">
         <v>54318</v>
       </c>
@@ -12645,6 +12864,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E230" t="inlineStr"/>
+      <c r="F230" t="inlineStr"/>
       <c r="G230" s="6" t="n">
         <v>50013</v>
       </c>
@@ -12692,6 +12913,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E231" t="inlineStr"/>
+      <c r="F231" t="inlineStr"/>
       <c r="G231" s="6" t="n">
         <v>66756</v>
       </c>
@@ -12739,6 +12962,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E232" t="inlineStr"/>
+      <c r="F232" t="inlineStr"/>
       <c r="G232" s="6" t="n">
         <v>62080</v>
       </c>
@@ -12786,6 +13011,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E233" t="inlineStr"/>
+      <c r="F233" t="inlineStr"/>
       <c r="G233" s="6" t="n">
         <v>58987</v>
       </c>
@@ -12833,6 +13060,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E234" t="inlineStr"/>
+      <c r="F234" t="inlineStr"/>
       <c r="G234" s="6" t="n">
         <v>51073</v>
       </c>
@@ -12880,6 +13109,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E235" t="inlineStr"/>
+      <c r="F235" t="inlineStr"/>
       <c r="G235" s="6" t="n">
         <v>53189</v>
       </c>
@@ -12927,6 +13158,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E236" t="inlineStr"/>
+      <c r="F236" t="inlineStr"/>
       <c r="G236" s="6" t="n">
         <v>67032</v>
       </c>
@@ -12974,6 +13207,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E237" t="inlineStr"/>
+      <c r="F237" t="inlineStr"/>
       <c r="G237" s="6" t="n">
         <v>63178</v>
       </c>
@@ -13021,6 +13256,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E238" t="inlineStr"/>
+      <c r="F238" t="inlineStr"/>
       <c r="G238" s="6" t="n">
         <v>54140</v>
       </c>
@@ -13068,6 +13305,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E239" t="inlineStr"/>
+      <c r="F239" t="inlineStr"/>
       <c r="G239" s="6" t="n">
         <v>71795</v>
       </c>
@@ -13115,6 +13354,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E240" t="inlineStr"/>
+      <c r="F240" t="inlineStr"/>
       <c r="G240" s="6" t="n">
         <v>69596</v>
       </c>
@@ -13162,6 +13403,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E241" t="inlineStr"/>
+      <c r="F241" t="inlineStr"/>
       <c r="G241" s="6" t="n">
         <v>73847</v>
       </c>
@@ -13209,6 +13452,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E242" t="inlineStr"/>
+      <c r="F242" t="inlineStr"/>
       <c r="G242" s="6" t="n">
         <v>84767</v>
       </c>
@@ -13256,6 +13501,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E243" t="inlineStr"/>
+      <c r="F243" t="inlineStr"/>
       <c r="G243" s="6" t="n">
         <v>70527</v>
       </c>
@@ -13303,6 +13550,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E244" t="inlineStr"/>
+      <c r="F244" t="inlineStr"/>
       <c r="G244" s="6" t="n">
         <v>71362</v>
       </c>
@@ -13350,6 +13599,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E245" t="inlineStr"/>
+      <c r="F245" t="inlineStr"/>
       <c r="G245" s="6" t="n">
         <v>77589</v>
       </c>
@@ -13397,6 +13648,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E246" t="inlineStr"/>
+      <c r="F246" t="inlineStr"/>
       <c r="G246" s="6" t="n">
         <v>89366</v>
       </c>
@@ -13444,6 +13697,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E247" t="inlineStr"/>
+      <c r="F247" t="inlineStr"/>
       <c r="G247" s="6" t="n">
         <v>93443</v>
       </c>
@@ -13491,6 +13746,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E248" t="inlineStr"/>
+      <c r="F248" t="inlineStr"/>
       <c r="G248" s="6" t="n">
         <v>100937</v>
       </c>
@@ -13538,6 +13795,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E249" t="inlineStr"/>
+      <c r="F249" t="inlineStr"/>
       <c r="G249" s="6" t="n">
         <v>101454</v>
       </c>
@@ -16057,25 +16316,19 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="E295" t="n">
-        <v>2500</v>
-      </c>
-      <c r="F295" t="inlineStr">
-        <is>
-          <t>price list 2019 (Price List India 2022-23.pdf)</t>
-        </is>
-      </c>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr"/>
+      <c r="F295" t="inlineStr"/>
       <c r="G295" s="6" t="n">
         <v>1205</v>
       </c>
       <c r="H295" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I295" s="3" t="n">
-        <v>2500</v>
+        <v>1550</v>
       </c>
       <c r="J295">
         <f>IF(I295&gt;0,CEILING(I295*(1-Policy!$B$13/100),IF(I295&lt;10000,50,100)),"")</f>
@@ -16116,11 +16369,11 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>2200</v>
+        <v>1800</v>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>price list 2019 (Price List India 2022-23.pdf)</t>
+          <t>product_list:market</t>
         </is>
       </c>
       <c r="G296" t="n">
@@ -16130,7 +16383,7 @@
         <v>0</v>
       </c>
       <c r="I296" s="3" t="n">
-        <v>2200</v>
+        <v>1800</v>
       </c>
       <c r="J296">
         <f>IF(I296&gt;0,CEILING(I296*(1-Policy!$B$13/100),IF(I296&lt;10000,50,100)),"")</f>
@@ -16280,6 +16533,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E299" t="inlineStr"/>
+      <c r="F299" t="inlineStr"/>
       <c r="G299" s="6" t="n">
         <v>5461</v>
       </c>
@@ -16327,6 +16582,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E300" t="inlineStr"/>
+      <c r="F300" t="inlineStr"/>
       <c r="G300" s="6" t="n">
         <v>5461</v>
       </c>
@@ -20432,11 +20689,11 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>15500</v>
+        <v>25000</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Paresh 25-09-2026, from WR costing sheets</t>
+          <t>confirmed by Paresh 24-09-2026</t>
         </is>
       </c>
       <c r="G62" t="n">
@@ -23498,6 +23755,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" s="6" t="n">
         <v>1200</v>
       </c>
@@ -23545,6 +23804,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" s="6" t="n">
         <v>1200</v>
       </c>
@@ -23592,6 +23853,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" s="6" t="n">
         <v>2200</v>
       </c>
@@ -23639,6 +23902,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" s="6" t="n">
         <v>1500</v>
       </c>
@@ -23686,6 +23951,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" s="6" t="n">
         <v>2600</v>
       </c>
@@ -23733,6 +24000,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" s="6" t="n">
         <v>1800</v>
       </c>
@@ -23780,6 +24049,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" s="6" t="n">
         <v>450</v>
       </c>
@@ -23827,6 +24098,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" s="6" t="n">
         <v>2400</v>
       </c>
@@ -23874,6 +24147,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" s="6" t="n">
         <v>900</v>
       </c>
@@ -23921,6 +24196,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" s="6" t="n">
         <v>250</v>
       </c>
@@ -23968,6 +24245,8 @@
           <t>on request</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" s="6" t="n">
         <v>0</v>
       </c>
@@ -24015,6 +24294,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" s="6" t="n">
         <v>350</v>
       </c>
@@ -24062,6 +24343,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" s="6" t="n">
         <v>600</v>
       </c>
@@ -24109,6 +24392,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" s="6" t="n">
         <v>900</v>
       </c>
@@ -24156,6 +24441,8 @@
           <t>on request</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" s="6" t="n">
         <v>0</v>
       </c>
@@ -24203,6 +24490,8 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" s="6" t="n">
         <v>6500</v>
       </c>
@@ -24250,6 +24539,8 @@
           <t>on request</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" s="6" t="n">
         <v>0</v>
       </c>
@@ -24422,6 +24713,7 @@
       <c r="L2" t="n">
         <v>21</v>
       </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -24472,6 +24764,7 @@
       <c r="L3" t="n">
         <v>21</v>
       </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -24522,6 +24815,7 @@
       <c r="L4" t="n">
         <v>21</v>
       </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -24572,6 +24866,7 @@
       <c r="L5" t="n">
         <v>21</v>
       </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -24622,6 +24917,7 @@
       <c r="L6" t="n">
         <v>21</v>
       </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -24672,6 +24968,7 @@
       <c r="L7" t="n">
         <v>21</v>
       </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -24722,6 +25019,7 @@
       <c r="L8" t="n">
         <v>21</v>
       </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -24772,6 +25070,7 @@
       <c r="L9" t="n">
         <v>21</v>
       </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -24822,6 +25121,7 @@
       <c r="L10" t="n">
         <v>21</v>
       </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -24872,6 +25172,7 @@
       <c r="L11" t="n">
         <v>21</v>
       </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -24922,6 +25223,7 @@
       <c r="L12" t="n">
         <v>21</v>
       </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -24972,6 +25274,7 @@
       <c r="L13" t="n">
         <v>21</v>
       </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -25022,6 +25325,7 @@
       <c r="L14" t="n">
         <v>21</v>
       </c>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -25072,6 +25376,7 @@
       <c r="L15" t="n">
         <v>21</v>
       </c>
+      <c r="M15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M15"/>
@@ -33335,6 +33640,9 @@
       <c r="D94" t="n">
         <v>1150</v>
       </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
       <c r="H94" s="3" t="n">
         <v>4</v>
       </c>
@@ -33412,6 +33720,9 @@
       <c r="D95" t="n">
         <v>1750</v>
       </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
       <c r="H95" s="3" t="n">
         <v>4</v>
       </c>
@@ -33489,6 +33800,9 @@
       <c r="D96" t="n">
         <v>2200</v>
       </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
       <c r="H96" s="3" t="n">
         <v>4</v>
       </c>
@@ -33566,6 +33880,9 @@
       <c r="D97" t="n">
         <v>2200</v>
       </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
       <c r="H97" s="3" t="n">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
Restore full ImpactCal + name fix, catalogue photos, delete buttons, file attach
</commit_message>
<xml_diff>
--- a/pricing/ImpactCal_Pricelist_2026-09.xlsx
+++ b/pricing/ImpactCal_Pricelist_2026-09.xlsx
@@ -475,8 +475,6 @@
           <t>ADONI TECH — ImpactCal global price list &amp; costing</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -489,20 +487,14 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>PRICING POLICY (agreed 23-24 Sep 2026)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -515,7 +507,6 @@
           <t>Highest price found in any of the 8 uploaded price lists is taken as-is (list price).</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -528,7 +519,6 @@
           <t>Cost model per series (price ~ k · Fs^a · stroke^b fitted on your own prices; median error 6 % crane, 9 % industrial) + negotiation margin below</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -541,7 +531,6 @@
           <t>Moulding cost + hardware + mould cost amortised, + margin over cost (parameters below; Rubber mounts sheet recalculates live)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -554,7 +543,6 @@
           <t>nearest ₹50 below ₹10,000, nearest ₹100 above (always up)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -567,12 +555,8 @@
           <t>list ÷ live INR/USD rate × (1 + export uplift); recomputed at quotation time; column here is indicative</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -811,7 +795,6 @@
           <t>8 / 4 / 1</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1044,8 +1027,6 @@
           <t>blue = estimated value</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1385,11 +1366,11 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>980</v>
+        <v>1100</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>product_list:market</t>
+          <t>price list 2019 (Price List India 2022-23.pdf)</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -1399,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="J6">
         <f>IF(I6&gt;0,CEILING(I6*(1-Policy!$B$13/100),IF(I6&lt;10000,50,100)),"")</f>
@@ -1659,8 +1640,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" s="6" t="n">
         <v>3669</v>
       </c>
@@ -2530,19 +2509,25 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>11000</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G27" s="6" t="n">
         <v>13156</v>
       </c>
       <c r="H27" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>16500</v>
+        <v>11000</v>
       </c>
       <c r="J27">
         <f>IF(I27&gt;0,CEILING(I27*(1-Policy!$B$13/100),IF(I27&lt;10000,50,100)),"")</f>
@@ -2579,19 +2564,25 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>12500</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G28" s="6" t="n">
         <v>15556</v>
       </c>
       <c r="H28" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>19500</v>
+        <v>12500</v>
       </c>
       <c r="J28">
         <f>IF(I28&gt;0,CEILING(I28*(1-Policy!$B$13/100),IF(I28&lt;10000,50,100)),"")</f>
@@ -2631,8 +2622,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" s="6" t="n">
         <v>22637</v>
       </c>
@@ -2680,8 +2669,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" s="6" t="n">
         <v>22711</v>
       </c>
@@ -2729,8 +2716,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" s="6" t="n">
         <v>30472</v>
       </c>
@@ -2778,8 +2763,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" s="6" t="n">
         <v>32765</v>
       </c>
@@ -2827,8 +2810,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" s="6" t="n">
         <v>35158</v>
       </c>
@@ -2876,8 +2857,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" s="6" t="n">
         <v>4638</v>
       </c>
@@ -2925,8 +2904,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
       <c r="G35" s="6" t="n">
         <v>4638</v>
       </c>
@@ -2974,8 +2951,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" s="6" t="n">
         <v>6578</v>
       </c>
@@ -3078,8 +3053,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" s="6" t="n">
         <v>8783</v>
       </c>
@@ -3127,8 +3100,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
       <c r="G39" s="6" t="n">
         <v>12227</v>
       </c>
@@ -3176,8 +3147,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
       <c r="G40" s="6" t="n">
         <v>14740</v>
       </c>
@@ -3225,8 +3194,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
       <c r="G41" s="6" t="n">
         <v>16533</v>
       </c>
@@ -3275,11 +3242,11 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1300</v>
+        <v>1400</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>product_list:b2b</t>
+          <t>price list 2019 (Price List India 2022-23.pdf)</t>
         </is>
       </c>
       <c r="G42" t="n">
@@ -3289,7 +3256,7 @@
         <v>0</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>1300</v>
+        <v>1400</v>
       </c>
       <c r="J42">
         <f>IF(I42&gt;0,CEILING(I42*(1-Policy!$B$13/100),IF(I42&lt;10000,50,100)),"")</f>
@@ -3330,11 +3297,11 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>2200</v>
+        <v>2400</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>product_list:market</t>
+          <t>price list 2019 (Price List India 2022-23.pdf)</t>
         </is>
       </c>
       <c r="G43" t="n">
@@ -3344,7 +3311,7 @@
         <v>0</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>2200</v>
+        <v>2400</v>
       </c>
       <c r="J43">
         <f>IF(I43&gt;0,CEILING(I43*(1-Policy!$B$13/100),IF(I43&lt;10000,50,100)),"")</f>
@@ -3494,8 +3461,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" s="6" t="n">
         <v>4235</v>
       </c>
@@ -4145,19 +4110,25 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G58" s="6" t="n">
         <v>7701</v>
       </c>
       <c r="H58" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>9650</v>
+        <v>8500</v>
       </c>
       <c r="J58">
         <f>IF(I58&gt;0,CEILING(I58*(1-Policy!$B$13/100),IF(I58&lt;10000,50,100)),"")</f>
@@ -4249,19 +4220,25 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>11800</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G60" s="6" t="n">
         <v>9296</v>
       </c>
       <c r="H60" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>11700</v>
+        <v>11800</v>
       </c>
       <c r="J60">
         <f>IF(I60&gt;0,CEILING(I60*(1-Policy!$B$13/100),IF(I60&lt;10000,50,100)),"")</f>
@@ -4298,19 +4275,25 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G61" s="6" t="n">
         <v>10378</v>
       </c>
       <c r="H61" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I61" s="3" t="n">
-        <v>13000</v>
+        <v>12000</v>
       </c>
       <c r="J61">
         <f>IF(I61&gt;0,CEILING(I61*(1-Policy!$B$13/100),IF(I61&lt;10000,50,100)),"")</f>
@@ -4347,19 +4330,25 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G62" s="6" t="n">
         <v>14212</v>
       </c>
       <c r="H62" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>17800</v>
+        <v>15000</v>
       </c>
       <c r="J62">
         <f>IF(I62&gt;0,CEILING(I62*(1-Policy!$B$13/100),IF(I62&lt;10000,50,100)),"")</f>
@@ -4396,19 +4385,25 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>17500</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G63" s="6" t="n">
         <v>16805</v>
       </c>
       <c r="H63" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>21100</v>
+        <v>17500</v>
       </c>
       <c r="J63">
         <f>IF(I63&gt;0,CEILING(I63*(1-Policy!$B$13/100),IF(I63&lt;10000,50,100)),"")</f>
@@ -4503,8 +4498,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
       <c r="G65" s="6" t="n">
         <v>40131</v>
       </c>
@@ -4549,19 +4542,25 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>44000</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G66" s="6" t="n">
         <v>32918</v>
       </c>
       <c r="H66" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>41200</v>
+        <v>44000</v>
       </c>
       <c r="J66">
         <f>IF(I66&gt;0,CEILING(I66*(1-Policy!$B$13/100),IF(I66&lt;10000,50,100)),"")</f>
@@ -4598,19 +4597,25 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>50000</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G67" s="6" t="n">
         <v>35395</v>
       </c>
       <c r="H67" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I67" s="3" t="n">
-        <v>44300</v>
+        <v>50000</v>
       </c>
       <c r="J67">
         <f>IF(I67&gt;0,CEILING(I67*(1-Policy!$B$13/100),IF(I67&lt;10000,50,100)),"")</f>
@@ -4647,19 +4652,25 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>55000</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>additional models 2018 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G68" s="6" t="n">
         <v>37981</v>
       </c>
       <c r="H68" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>47500</v>
+        <v>55000</v>
       </c>
       <c r="J68">
         <f>IF(I68&gt;0,CEILING(I68*(1-Policy!$B$13/100),IF(I68&lt;10000,50,100)),"")</f>
@@ -4919,8 +4930,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" s="6" t="n">
         <v>20689</v>
       </c>
@@ -5353,8 +5362,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
       <c r="G81" s="6" t="n">
         <v>26890</v>
       </c>
@@ -5897,8 +5904,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
-      <c r="F91" t="inlineStr"/>
       <c r="G91" s="6" t="n">
         <v>52785</v>
       </c>
@@ -5946,8 +5951,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="inlineStr"/>
       <c r="G92" s="6" t="n">
         <v>60795</v>
       </c>
@@ -5995,8 +5998,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
-      <c r="F93" t="inlineStr"/>
       <c r="G93" s="6" t="n">
         <v>68832</v>
       </c>
@@ -6264,8 +6265,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr"/>
       <c r="G98" s="6" t="n">
         <v>58913</v>
       </c>
@@ -6313,8 +6312,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr"/>
       <c r="G99" s="6" t="n">
         <v>69090</v>
       </c>
@@ -6527,8 +6524,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr"/>
       <c r="G103" s="6" t="n">
         <v>70653</v>
       </c>
@@ -6741,8 +6736,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr"/>
       <c r="G107" s="6" t="n">
         <v>81211</v>
       </c>
@@ -6955,8 +6948,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
       <c r="G111" s="6" t="n">
         <v>73543</v>
       </c>
@@ -7059,8 +7050,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
       <c r="G113" s="6" t="n">
         <v>85653</v>
       </c>
@@ -7493,8 +7482,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr"/>
       <c r="G121" s="6" t="n">
         <v>89371</v>
       </c>
@@ -7542,8 +7529,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" s="6" t="n">
         <v>80189</v>
       </c>
@@ -7701,8 +7686,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr"/>
       <c r="G125" s="6" t="n">
         <v>81294</v>
       </c>
@@ -7805,8 +7788,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr"/>
       <c r="G127" s="6" t="n">
         <v>94259</v>
       </c>
@@ -7909,8 +7890,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
-      <c r="F129" t="inlineStr"/>
       <c r="G129" s="6" t="n">
         <v>80100</v>
       </c>
@@ -7958,8 +7937,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
-      <c r="F130" t="inlineStr"/>
       <c r="G130" s="6" t="n">
         <v>79673</v>
       </c>
@@ -8007,8 +7984,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
-      <c r="F131" t="inlineStr"/>
       <c r="G131" s="6" t="n">
         <v>99666</v>
       </c>
@@ -8056,8 +8031,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
-      <c r="F132" t="inlineStr"/>
       <c r="G132" s="6" t="n">
         <v>106423</v>
       </c>
@@ -8105,8 +8078,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
-      <c r="F133" t="inlineStr"/>
       <c r="G133" s="6" t="n">
         <v>112858</v>
       </c>
@@ -8209,8 +8180,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
-      <c r="F135" t="inlineStr"/>
       <c r="G135" s="6" t="n">
         <v>29935</v>
       </c>
@@ -8258,8 +8227,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
-      <c r="F136" t="inlineStr"/>
       <c r="G136" s="6" t="n">
         <v>31513</v>
       </c>
@@ -8307,8 +8274,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
-      <c r="F137" t="inlineStr"/>
       <c r="G137" s="6" t="n">
         <v>42694</v>
       </c>
@@ -8356,8 +8321,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
-      <c r="F138" t="inlineStr"/>
       <c r="G138" s="6" t="n">
         <v>49521</v>
       </c>
@@ -8405,8 +8368,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
-      <c r="F139" t="inlineStr"/>
       <c r="G139" s="6" t="n">
         <v>45237</v>
       </c>
@@ -8454,8 +8415,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
-      <c r="F140" t="inlineStr"/>
       <c r="G140" s="6" t="n">
         <v>55448</v>
       </c>
@@ -8503,8 +8462,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
-      <c r="F141" t="inlineStr"/>
       <c r="G141" s="6" t="n">
         <v>15625</v>
       </c>
@@ -8552,8 +8509,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
-      <c r="F142" t="inlineStr"/>
       <c r="G142" s="6" t="n">
         <v>17980</v>
       </c>
@@ -8601,8 +8556,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
-      <c r="F143" t="inlineStr"/>
       <c r="G143" s="6" t="n">
         <v>19750</v>
       </c>
@@ -8650,8 +8603,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr"/>
-      <c r="F144" t="inlineStr"/>
       <c r="G144" s="6" t="n">
         <v>27713</v>
       </c>
@@ -8699,8 +8650,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr"/>
       <c r="G145" s="6" t="n">
         <v>21214</v>
       </c>
@@ -8748,8 +8697,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr"/>
-      <c r="F146" t="inlineStr"/>
       <c r="G146" s="6" t="n">
         <v>32461</v>
       </c>
@@ -8797,8 +8744,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr"/>
-      <c r="F147" t="inlineStr"/>
       <c r="G147" s="6" t="n">
         <v>30749</v>
       </c>
@@ -8846,8 +8791,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
-      <c r="F148" t="inlineStr"/>
       <c r="G148" s="6" t="n">
         <v>22335</v>
       </c>
@@ -8895,8 +8838,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr"/>
-      <c r="F149" t="inlineStr"/>
       <c r="G149" s="6" t="n">
         <v>35819</v>
       </c>
@@ -8944,8 +8885,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
-      <c r="F150" t="inlineStr"/>
       <c r="G150" s="6" t="n">
         <v>27425</v>
       </c>
@@ -8993,8 +8932,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr"/>
-      <c r="F151" t="inlineStr"/>
       <c r="G151" s="6" t="n">
         <v>23369</v>
       </c>
@@ -9042,8 +8979,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr"/>
-      <c r="F152" t="inlineStr"/>
       <c r="G152" s="6" t="n">
         <v>23976</v>
       </c>
@@ -9091,8 +9026,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr"/>
-      <c r="F153" t="inlineStr"/>
       <c r="G153" s="6" t="n">
         <v>29404</v>
       </c>
@@ -9140,8 +9073,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr"/>
-      <c r="F154" t="inlineStr"/>
       <c r="G154" s="6" t="n">
         <v>24434</v>
       </c>
@@ -9189,8 +9120,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
-      <c r="F155" t="inlineStr"/>
       <c r="G155" s="6" t="n">
         <v>34635</v>
       </c>
@@ -9238,8 +9167,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr"/>
-      <c r="F156" t="inlineStr"/>
       <c r="G156" s="6" t="n">
         <v>24670</v>
       </c>
@@ -9287,8 +9214,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr"/>
-      <c r="F157" t="inlineStr"/>
       <c r="G157" s="6" t="n">
         <v>38300</v>
       </c>
@@ -9336,8 +9261,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr"/>
-      <c r="F158" t="inlineStr"/>
       <c r="G158" s="6" t="n">
         <v>24867</v>
       </c>
@@ -9385,8 +9308,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr"/>
-      <c r="F159" t="inlineStr"/>
       <c r="G159" s="6" t="n">
         <v>31172</v>
       </c>
@@ -9434,8 +9355,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr"/>
-      <c r="F160" t="inlineStr"/>
       <c r="G160" s="6" t="n">
         <v>25070</v>
       </c>
@@ -9483,8 +9402,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E161" t="inlineStr"/>
-      <c r="F161" t="inlineStr"/>
       <c r="G161" s="6" t="n">
         <v>42121</v>
       </c>
@@ -9532,8 +9449,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr"/>
-      <c r="F162" t="inlineStr"/>
       <c r="G162" s="6" t="n">
         <v>25112</v>
       </c>
@@ -9581,8 +9496,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr"/>
-      <c r="F163" t="inlineStr"/>
       <c r="G163" s="6" t="n">
         <v>32430</v>
       </c>
@@ -9630,8 +9543,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr"/>
-      <c r="F164" t="inlineStr"/>
       <c r="G164" s="6" t="n">
         <v>37139</v>
       </c>
@@ -9679,8 +9590,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr"/>
-      <c r="F165" t="inlineStr"/>
       <c r="G165" s="6" t="n">
         <v>25264</v>
       </c>
@@ -9728,8 +9637,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr"/>
-      <c r="F166" t="inlineStr"/>
       <c r="G166" s="6" t="n">
         <v>33063</v>
       </c>
@@ -9777,8 +9684,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr"/>
-      <c r="F167" t="inlineStr"/>
       <c r="G167" s="6" t="n">
         <v>42077</v>
       </c>
@@ -9826,8 +9731,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E168" t="inlineStr"/>
-      <c r="F168" t="inlineStr"/>
       <c r="G168" s="6" t="n">
         <v>33717</v>
       </c>
@@ -9875,8 +9778,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E169" t="inlineStr"/>
-      <c r="F169" t="inlineStr"/>
       <c r="G169" s="6" t="n">
         <v>38513</v>
       </c>
@@ -9924,8 +9825,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E170" t="inlineStr"/>
-      <c r="F170" t="inlineStr"/>
       <c r="G170" s="6" t="n">
         <v>46129</v>
       </c>
@@ -9973,8 +9872,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E171" t="inlineStr"/>
-      <c r="F171" t="inlineStr"/>
       <c r="G171" s="6" t="n">
         <v>34304</v>
       </c>
@@ -10022,8 +9919,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E172" t="inlineStr"/>
-      <c r="F172" t="inlineStr"/>
       <c r="G172" s="6" t="n">
         <v>39761</v>
       </c>
@@ -10071,8 +9966,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E173" t="inlineStr"/>
-      <c r="F173" t="inlineStr"/>
       <c r="G173" s="6" t="n">
         <v>44687</v>
       </c>
@@ -10120,8 +10013,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr"/>
-      <c r="F174" t="inlineStr"/>
       <c r="G174" s="6" t="n">
         <v>34832</v>
       </c>
@@ -10169,8 +10060,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr"/>
-      <c r="F175" t="inlineStr"/>
       <c r="G175" s="6" t="n">
         <v>35928</v>
       </c>
@@ -10218,8 +10107,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E176" t="inlineStr"/>
-      <c r="F176" t="inlineStr"/>
       <c r="G176" s="6" t="n">
         <v>46027</v>
       </c>
@@ -10267,8 +10154,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E177" t="inlineStr"/>
-      <c r="F177" t="inlineStr"/>
       <c r="G177" s="6" t="n">
         <v>49530</v>
       </c>
@@ -10316,8 +10201,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr"/>
-      <c r="F178" t="inlineStr"/>
       <c r="G178" s="6" t="n">
         <v>42595</v>
       </c>
@@ -10365,8 +10248,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr"/>
-      <c r="F179" t="inlineStr"/>
       <c r="G179" s="6" t="n">
         <v>36962</v>
       </c>
@@ -10414,8 +10295,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr"/>
-      <c r="F180" t="inlineStr"/>
       <c r="G180" s="6" t="n">
         <v>43498</v>
       </c>
@@ -10463,8 +10342,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr"/>
-      <c r="F181" t="inlineStr"/>
       <c r="G181" s="6" t="n">
         <v>35830</v>
       </c>
@@ -10512,8 +10389,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr"/>
-      <c r="F182" t="inlineStr"/>
       <c r="G182" s="6" t="n">
         <v>47326</v>
       </c>
@@ -10561,8 +10436,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr"/>
-      <c r="F183" t="inlineStr"/>
       <c r="G183" s="6" t="n">
         <v>52098</v>
       </c>
@@ -10610,8 +10483,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr"/>
-      <c r="F184" t="inlineStr"/>
       <c r="G184" s="6" t="n">
         <v>44353</v>
       </c>
@@ -10659,8 +10530,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E185" t="inlineStr"/>
-      <c r="F185" t="inlineStr"/>
       <c r="G185" s="6" t="n">
         <v>45164</v>
       </c>
@@ -10708,8 +10577,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E186" t="inlineStr"/>
-      <c r="F186" t="inlineStr"/>
       <c r="G186" s="6" t="n">
         <v>49586</v>
       </c>
@@ -10757,8 +10624,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E187" t="inlineStr"/>
-      <c r="F187" t="inlineStr"/>
       <c r="G187" s="6" t="n">
         <v>54439</v>
       </c>
@@ -10806,8 +10671,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E188" t="inlineStr"/>
-      <c r="F188" t="inlineStr"/>
       <c r="G188" s="6" t="n">
         <v>46646</v>
       </c>
@@ -10855,8 +10718,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E189" t="inlineStr"/>
-      <c r="F189" t="inlineStr"/>
       <c r="G189" s="6" t="n">
         <v>41784</v>
       </c>
@@ -10904,8 +10765,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E190" t="inlineStr"/>
-      <c r="F190" t="inlineStr"/>
       <c r="G190" s="6" t="n">
         <v>40599</v>
       </c>
@@ -10953,8 +10812,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr"/>
-      <c r="F191" t="inlineStr"/>
       <c r="G191" s="6" t="n">
         <v>41080</v>
       </c>
@@ -11002,8 +10859,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E192" t="inlineStr"/>
-      <c r="F192" t="inlineStr"/>
       <c r="G192" s="6" t="n">
         <v>48023</v>
       </c>
@@ -11051,8 +10906,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E193" t="inlineStr"/>
-      <c r="F193" t="inlineStr"/>
       <c r="G193" s="6" t="n">
         <v>53650</v>
       </c>
@@ -11100,8 +10953,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E194" t="inlineStr"/>
-      <c r="F194" t="inlineStr"/>
       <c r="G194" s="6" t="n">
         <v>58216</v>
       </c>
@@ -11149,8 +11000,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E195" t="inlineStr"/>
-      <c r="F195" t="inlineStr"/>
       <c r="G195" s="6" t="n">
         <v>41168</v>
       </c>
@@ -11198,8 +11047,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E196" t="inlineStr"/>
-      <c r="F196" t="inlineStr"/>
       <c r="G196" s="6" t="n">
         <v>49268</v>
       </c>
@@ -11247,8 +11094,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E197" t="inlineStr"/>
-      <c r="F197" t="inlineStr"/>
       <c r="G197" s="6" t="n">
         <v>55239</v>
       </c>
@@ -11296,8 +11141,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E198" t="inlineStr"/>
-      <c r="F198" t="inlineStr"/>
       <c r="G198" s="6" t="n">
         <v>50893</v>
       </c>
@@ -11345,8 +11188,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E199" t="inlineStr"/>
-      <c r="F199" t="inlineStr"/>
       <c r="G199" s="6" t="n">
         <v>61426</v>
       </c>
@@ -11394,8 +11235,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E200" t="inlineStr"/>
-      <c r="F200" t="inlineStr"/>
       <c r="G200" s="6" t="n">
         <v>56693</v>
       </c>
@@ -11443,8 +11282,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr"/>
-      <c r="F201" t="inlineStr"/>
       <c r="G201" s="6" t="n">
         <v>51435</v>
       </c>
@@ -11492,8 +11329,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr"/>
-      <c r="F202" t="inlineStr"/>
       <c r="G202" s="6" t="n">
         <v>58064</v>
       </c>
@@ -11541,8 +11376,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E203" t="inlineStr"/>
-      <c r="F203" t="inlineStr"/>
       <c r="G203" s="6" t="n">
         <v>51967</v>
       </c>
@@ -11590,8 +11423,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E204" t="inlineStr"/>
-      <c r="F204" t="inlineStr"/>
       <c r="G204" s="6" t="n">
         <v>64157</v>
       </c>
@@ -11639,8 +11470,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E205" t="inlineStr"/>
-      <c r="F205" t="inlineStr"/>
       <c r="G205" s="6" t="n">
         <v>52150</v>
       </c>
@@ -11688,8 +11517,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E206" t="inlineStr"/>
-      <c r="F206" t="inlineStr"/>
       <c r="G206" s="6" t="n">
         <v>59346</v>
       </c>
@@ -11737,8 +11564,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E207" t="inlineStr"/>
-      <c r="F207" t="inlineStr"/>
       <c r="G207" s="6" t="n">
         <v>52495</v>
       </c>
@@ -11786,8 +11611,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr"/>
-      <c r="F208" t="inlineStr"/>
       <c r="G208" s="6" t="n">
         <v>66481</v>
       </c>
@@ -11835,8 +11658,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr"/>
-      <c r="F209" t="inlineStr"/>
       <c r="G209" s="6" t="n">
         <v>60346</v>
       </c>
@@ -11884,8 +11705,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E210" t="inlineStr"/>
-      <c r="F210" t="inlineStr"/>
       <c r="G210" s="6" t="n">
         <v>52676</v>
       </c>
@@ -11933,8 +11752,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E211" t="inlineStr"/>
-      <c r="F211" t="inlineStr"/>
       <c r="G211" s="6" t="n">
         <v>53397</v>
       </c>
@@ -11982,8 +11799,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E212" t="inlineStr"/>
-      <c r="F212" t="inlineStr"/>
       <c r="G212" s="6" t="n">
         <v>67853</v>
       </c>
@@ -12031,8 +11846,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E213" t="inlineStr"/>
-      <c r="F213" t="inlineStr"/>
       <c r="G213" s="6" t="n">
         <v>61371</v>
       </c>
@@ -12080,8 +11893,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E214" t="inlineStr"/>
-      <c r="F214" t="inlineStr"/>
       <c r="G214" s="6" t="n">
         <v>69157</v>
       </c>
@@ -12129,8 +11940,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E215" t="inlineStr"/>
-      <c r="F215" t="inlineStr"/>
       <c r="G215" s="6" t="n">
         <v>61909</v>
       </c>
@@ -12178,8 +11987,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E216" t="inlineStr"/>
-      <c r="F216" t="inlineStr"/>
       <c r="G216" s="6" t="n">
         <v>70220</v>
       </c>
@@ -12227,8 +12034,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E217" t="inlineStr"/>
-      <c r="F217" t="inlineStr"/>
       <c r="G217" s="6" t="n">
         <v>71273</v>
       </c>
@@ -12276,8 +12081,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E218" t="inlineStr"/>
-      <c r="F218" t="inlineStr"/>
       <c r="G218" s="6" t="n">
         <v>16373</v>
       </c>
@@ -12325,8 +12128,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E219" t="inlineStr"/>
-      <c r="F219" t="inlineStr"/>
       <c r="G219" s="6" t="n">
         <v>19173</v>
       </c>
@@ -12374,8 +12175,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr"/>
-      <c r="F220" t="inlineStr"/>
       <c r="G220" s="6" t="n">
         <v>24869</v>
       </c>
@@ -12423,8 +12222,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E221" t="inlineStr"/>
-      <c r="F221" t="inlineStr"/>
       <c r="G221" s="6" t="n">
         <v>30450</v>
       </c>
@@ -12472,8 +12269,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E222" t="inlineStr"/>
-      <c r="F222" t="inlineStr"/>
       <c r="G222" s="6" t="n">
         <v>29342</v>
       </c>
@@ -12521,8 +12316,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr"/>
-      <c r="F223" t="inlineStr"/>
       <c r="G223" s="6" t="n">
         <v>35927</v>
       </c>
@@ -12570,8 +12363,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr"/>
-      <c r="F224" t="inlineStr"/>
       <c r="G224" s="6" t="n">
         <v>39577</v>
       </c>
@@ -12619,8 +12410,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E225" t="inlineStr"/>
-      <c r="F225" t="inlineStr"/>
       <c r="G225" s="6" t="n">
         <v>46038</v>
       </c>
@@ -12668,8 +12457,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E226" t="inlineStr"/>
-      <c r="F226" t="inlineStr"/>
       <c r="G226" s="6" t="n">
         <v>42389</v>
       </c>
@@ -12717,8 +12504,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E227" t="inlineStr"/>
-      <c r="F227" t="inlineStr"/>
       <c r="G227" s="6" t="n">
         <v>50476</v>
       </c>
@@ -12766,8 +12551,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E228" t="inlineStr"/>
-      <c r="F228" t="inlineStr"/>
       <c r="G228" s="6" t="n">
         <v>62169</v>
       </c>
@@ -12815,8 +12598,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E229" t="inlineStr"/>
-      <c r="F229" t="inlineStr"/>
       <c r="G229" s="6" t="n">
         <v>54318</v>
       </c>
@@ -12864,8 +12645,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E230" t="inlineStr"/>
-      <c r="F230" t="inlineStr"/>
       <c r="G230" s="6" t="n">
         <v>50013</v>
       </c>
@@ -12913,8 +12692,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E231" t="inlineStr"/>
-      <c r="F231" t="inlineStr"/>
       <c r="G231" s="6" t="n">
         <v>66756</v>
       </c>
@@ -12962,8 +12739,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E232" t="inlineStr"/>
-      <c r="F232" t="inlineStr"/>
       <c r="G232" s="6" t="n">
         <v>62080</v>
       </c>
@@ -13011,8 +12786,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E233" t="inlineStr"/>
-      <c r="F233" t="inlineStr"/>
       <c r="G233" s="6" t="n">
         <v>58987</v>
       </c>
@@ -13060,8 +12833,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E234" t="inlineStr"/>
-      <c r="F234" t="inlineStr"/>
       <c r="G234" s="6" t="n">
         <v>51073</v>
       </c>
@@ -13109,8 +12880,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E235" t="inlineStr"/>
-      <c r="F235" t="inlineStr"/>
       <c r="G235" s="6" t="n">
         <v>53189</v>
       </c>
@@ -13158,8 +12927,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr"/>
-      <c r="F236" t="inlineStr"/>
       <c r="G236" s="6" t="n">
         <v>67032</v>
       </c>
@@ -13207,8 +12974,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E237" t="inlineStr"/>
-      <c r="F237" t="inlineStr"/>
       <c r="G237" s="6" t="n">
         <v>63178</v>
       </c>
@@ -13256,8 +13021,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E238" t="inlineStr"/>
-      <c r="F238" t="inlineStr"/>
       <c r="G238" s="6" t="n">
         <v>54140</v>
       </c>
@@ -13305,8 +13068,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E239" t="inlineStr"/>
-      <c r="F239" t="inlineStr"/>
       <c r="G239" s="6" t="n">
         <v>71795</v>
       </c>
@@ -13354,8 +13115,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E240" t="inlineStr"/>
-      <c r="F240" t="inlineStr"/>
       <c r="G240" s="6" t="n">
         <v>69596</v>
       </c>
@@ -13403,8 +13162,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E241" t="inlineStr"/>
-      <c r="F241" t="inlineStr"/>
       <c r="G241" s="6" t="n">
         <v>73847</v>
       </c>
@@ -13452,8 +13209,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E242" t="inlineStr"/>
-      <c r="F242" t="inlineStr"/>
       <c r="G242" s="6" t="n">
         <v>84767</v>
       </c>
@@ -13501,8 +13256,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E243" t="inlineStr"/>
-      <c r="F243" t="inlineStr"/>
       <c r="G243" s="6" t="n">
         <v>70527</v>
       </c>
@@ -13550,8 +13303,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr"/>
-      <c r="F244" t="inlineStr"/>
       <c r="G244" s="6" t="n">
         <v>71362</v>
       </c>
@@ -13599,8 +13350,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E245" t="inlineStr"/>
-      <c r="F245" t="inlineStr"/>
       <c r="G245" s="6" t="n">
         <v>77589</v>
       </c>
@@ -13648,8 +13397,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E246" t="inlineStr"/>
-      <c r="F246" t="inlineStr"/>
       <c r="G246" s="6" t="n">
         <v>89366</v>
       </c>
@@ -13697,8 +13444,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E247" t="inlineStr"/>
-      <c r="F247" t="inlineStr"/>
       <c r="G247" s="6" t="n">
         <v>93443</v>
       </c>
@@ -13746,8 +13491,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E248" t="inlineStr"/>
-      <c r="F248" t="inlineStr"/>
       <c r="G248" s="6" t="n">
         <v>100937</v>
       </c>
@@ -13795,8 +13538,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E249" t="inlineStr"/>
-      <c r="F249" t="inlineStr"/>
       <c r="G249" s="6" t="n">
         <v>101454</v>
       </c>
@@ -16316,19 +16057,25 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="E295" t="inlineStr"/>
-      <c r="F295" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>price list 2019 (Price List India 2022-23.pdf)</t>
+        </is>
+      </c>
       <c r="G295" s="6" t="n">
         <v>1205</v>
       </c>
       <c r="H295" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I295" s="3" t="n">
-        <v>1550</v>
+        <v>2500</v>
       </c>
       <c r="J295">
         <f>IF(I295&gt;0,CEILING(I295*(1-Policy!$B$13/100),IF(I295&lt;10000,50,100)),"")</f>
@@ -16369,11 +16116,11 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>1800</v>
+        <v>2200</v>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>product_list:market</t>
+          <t>price list 2019 (Price List India 2022-23.pdf)</t>
         </is>
       </c>
       <c r="G296" t="n">
@@ -16383,7 +16130,7 @@
         <v>0</v>
       </c>
       <c r="I296" s="3" t="n">
-        <v>1800</v>
+        <v>2200</v>
       </c>
       <c r="J296">
         <f>IF(I296&gt;0,CEILING(I296*(1-Policy!$B$13/100),IF(I296&lt;10000,50,100)),"")</f>
@@ -16533,8 +16280,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E299" t="inlineStr"/>
-      <c r="F299" t="inlineStr"/>
       <c r="G299" s="6" t="n">
         <v>5461</v>
       </c>
@@ -16582,8 +16327,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E300" t="inlineStr"/>
-      <c r="F300" t="inlineStr"/>
       <c r="G300" s="6" t="n">
         <v>5461</v>
       </c>
@@ -20689,11 +20432,11 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>25000</v>
+        <v>15500</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>confirmed by Paresh 24-09-2026</t>
+          <t>Paresh 25-09-2026, from WR costing sheets</t>
         </is>
       </c>
       <c r="G62" t="n">
@@ -23755,8 +23498,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" s="6" t="n">
         <v>1200</v>
       </c>
@@ -23804,8 +23545,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" s="6" t="n">
         <v>1200</v>
       </c>
@@ -23853,8 +23592,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" s="6" t="n">
         <v>2200</v>
       </c>
@@ -23902,8 +23639,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" s="6" t="n">
         <v>1500</v>
       </c>
@@ -23951,8 +23686,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" s="6" t="n">
         <v>2600</v>
       </c>
@@ -24000,8 +23733,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" s="6" t="n">
         <v>1800</v>
       </c>
@@ -24049,8 +23780,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" s="6" t="n">
         <v>450</v>
       </c>
@@ -24098,8 +23827,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" s="6" t="n">
         <v>2400</v>
       </c>
@@ -24147,8 +23874,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" s="6" t="n">
         <v>900</v>
       </c>
@@ -24196,8 +23921,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" s="6" t="n">
         <v>250</v>
       </c>
@@ -24245,8 +23968,6 @@
           <t>on request</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" s="6" t="n">
         <v>0</v>
       </c>
@@ -24294,8 +24015,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" s="6" t="n">
         <v>350</v>
       </c>
@@ -24343,8 +24062,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" s="6" t="n">
         <v>600</v>
       </c>
@@ -24392,8 +24109,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" s="6" t="n">
         <v>900</v>
       </c>
@@ -24441,8 +24156,6 @@
           <t>on request</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" s="6" t="n">
         <v>0</v>
       </c>
@@ -24490,8 +24203,6 @@
           <t>model</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" s="6" t="n">
         <v>6500</v>
       </c>
@@ -24539,8 +24250,6 @@
           <t>on request</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" s="6" t="n">
         <v>0</v>
       </c>
@@ -24713,7 +24422,6 @@
       <c r="L2" t="n">
         <v>21</v>
       </c>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -24764,7 +24472,6 @@
       <c r="L3" t="n">
         <v>21</v>
       </c>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -24815,7 +24522,6 @@
       <c r="L4" t="n">
         <v>21</v>
       </c>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -24866,7 +24572,6 @@
       <c r="L5" t="n">
         <v>21</v>
       </c>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -24917,7 +24622,6 @@
       <c r="L6" t="n">
         <v>21</v>
       </c>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -24968,7 +24672,6 @@
       <c r="L7" t="n">
         <v>21</v>
       </c>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -25019,7 +24722,6 @@
       <c r="L8" t="n">
         <v>21</v>
       </c>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -25070,7 +24772,6 @@
       <c r="L9" t="n">
         <v>21</v>
       </c>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -25121,7 +24822,6 @@
       <c r="L10" t="n">
         <v>21</v>
       </c>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -25172,7 +24872,6 @@
       <c r="L11" t="n">
         <v>21</v>
       </c>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -25223,7 +24922,6 @@
       <c r="L12" t="n">
         <v>21</v>
       </c>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -25274,7 +24972,6 @@
       <c r="L13" t="n">
         <v>21</v>
       </c>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -25325,7 +25022,6 @@
       <c r="L14" t="n">
         <v>21</v>
       </c>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -25376,7 +25072,6 @@
       <c r="L15" t="n">
         <v>21</v>
       </c>
-      <c r="M15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M15"/>
@@ -33640,9 +33335,6 @@
       <c r="D94" t="n">
         <v>1150</v>
       </c>
-      <c r="E94" t="inlineStr"/>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" s="3" t="n">
         <v>4</v>
       </c>
@@ -33720,9 +33412,6 @@
       <c r="D95" t="n">
         <v>1750</v>
       </c>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
-      <c r="G95" t="inlineStr"/>
       <c r="H95" s="3" t="n">
         <v>4</v>
       </c>
@@ -33800,9 +33489,6 @@
       <c r="D96" t="n">
         <v>2200</v>
       </c>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
       <c r="H96" s="3" t="n">
         <v>4</v>
       </c>
@@ -33880,9 +33566,6 @@
       <c r="D97" t="n">
         <v>2200</v>
       </c>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
       <c r="H97" s="3" t="n">
         <v>4</v>
       </c>

</xml_diff>